<commit_message>
refactor: extract agenda logic to core.agenda
- Moved agenda day/date resolution, time parsing, and interval debug logic into core/agenda.py
- Updated clubal.py to delegate agenda computation while preserving the UI card format
- Kept CLUBAL_DEBUG_AGENDA diagnostics and cross-midnight handling
- Reduced domain logic inside clubal.py to improve separation between UI and orchestration
</commit_message>
<xml_diff>
--- a/grade.xlsx
+++ b/grade.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrativo\Desktop\Guilherme\Projeto_CLUBAL\CLUBAL\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrativo\Documents\GitHub\clubal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EB665C6-2725-4A70-88EA-F7FC81BFDF72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F8AC58B-4057-4A83-BC40-046A4FDE9636}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,7 +18,6 @@
     <sheet name="Nao_Aquaticos" sheetId="8" r:id="rId3"/>
     <sheet name="Vagas" sheetId="9" r:id="rId4"/>
     <sheet name="CLUBAL" sheetId="2" r:id="rId5"/>
-    <sheet name="test" sheetId="11" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="531" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="110">
   <si>
     <t>AULAS COLETIVAS</t>
   </si>
@@ -386,15 +385,6 @@
     <t>Amanda</t>
   </si>
   <si>
-    <t>Guilherme</t>
-  </si>
-  <si>
-    <t>Ludmila</t>
-  </si>
-  <si>
-    <t>Natasha</t>
-  </si>
-  <si>
     <t>MENOR</t>
   </si>
   <si>
@@ -408,15 +398,6 @@
   </si>
   <si>
     <t>Voleibol</t>
-  </si>
-  <si>
-    <t>Psicomotricidade</t>
-  </si>
-  <si>
-    <t>Futsal</t>
-  </si>
-  <si>
-    <t>Hidroginástica</t>
   </si>
 </sst>
 </file>
@@ -1518,40 +1499,19 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="20" fontId="5" fillId="9" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="9" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="2" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="8" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="8" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="2" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="20" fontId="5" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1560,16 +1520,34 @@
     <xf numFmtId="20" fontId="5" fillId="2" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="20" fontId="5" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="20" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="20" fontId="5" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="20" fontId="5" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="9" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1584,8 +1562,11 @@
     <xf numFmtId="0" fontId="5" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="20" fontId="5" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="2" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="20" fontId="5" fillId="9" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1593,43 +1574,43 @@
     <xf numFmtId="20" fontId="5" fillId="9" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="20" fontId="5" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="9" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="20" fontId="5" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="8" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="8" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="9" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="9" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="2" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1659,6 +1640,81 @@
     <xf numFmtId="0" fontId="5" fillId="9" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="7" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
@@ -1684,81 +1740,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="7" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2853,7 +2834,7 @@
       <c r="B4" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="C4" s="150" t="s">
+      <c r="C4" s="117" t="s">
         <v>24</v>
       </c>
       <c r="D4" s="114"/>
@@ -2865,23 +2846,23 @@
         <v>4</v>
       </c>
       <c r="H4" s="114"/>
-      <c r="I4" s="153" t="s">
+      <c r="I4" s="120" t="s">
         <v>5</v>
       </c>
-      <c r="J4" s="154"/>
-      <c r="K4" s="151" t="s">
+      <c r="J4" s="121"/>
+      <c r="K4" s="118" t="s">
         <v>6</v>
       </c>
-      <c r="L4" s="152"/>
-      <c r="M4" s="151" t="s">
+      <c r="L4" s="119"/>
+      <c r="M4" s="118" t="s">
         <v>35</v>
       </c>
-      <c r="N4" s="152"/>
+      <c r="N4" s="119"/>
       <c r="O4" s="2"/>
     </row>
     <row r="5" spans="1:15" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2"/>
-      <c r="B5" s="137" t="s">
+      <c r="B5" s="136" t="s">
         <v>22</v>
       </c>
       <c r="C5" s="140" t="s">
@@ -2912,15 +2893,15 @@
       <c r="L5" s="41">
         <v>0.45833333333333331</v>
       </c>
-      <c r="M5" s="125"/>
-      <c r="N5" s="126"/>
+      <c r="M5" s="145"/>
+      <c r="N5" s="146"/>
       <c r="O5" s="2"/>
     </row>
     <row r="6" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A6" s="2"/>
-      <c r="B6" s="138"/>
-      <c r="C6" s="142"/>
-      <c r="D6" s="143"/>
+      <c r="B6" s="137"/>
+      <c r="C6" s="128"/>
+      <c r="D6" s="129"/>
       <c r="E6" s="45">
         <v>0.73958333333333337</v>
       </c>
@@ -2937,17 +2918,17 @@
       </c>
       <c r="K6" s="45"/>
       <c r="L6" s="46"/>
-      <c r="M6" s="117"/>
-      <c r="N6" s="118"/>
+      <c r="M6" s="147"/>
+      <c r="N6" s="148"/>
       <c r="O6" s="2"/>
     </row>
     <row r="7" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
-      <c r="B7" s="138"/>
-      <c r="C7" s="142" t="s">
+      <c r="B7" s="137"/>
+      <c r="C7" s="128" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="143"/>
+      <c r="D7" s="129"/>
       <c r="E7" s="40">
         <v>0.42708333333333331</v>
       </c>
@@ -2964,15 +2945,15 @@
       </c>
       <c r="K7" s="40"/>
       <c r="L7" s="41"/>
-      <c r="M7" s="125"/>
-      <c r="N7" s="126"/>
+      <c r="M7" s="145"/>
+      <c r="N7" s="146"/>
       <c r="O7" s="2"/>
     </row>
     <row r="8" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A8" s="2"/>
-      <c r="B8" s="138"/>
-      <c r="C8" s="142"/>
-      <c r="D8" s="143"/>
+      <c r="B8" s="137"/>
+      <c r="C8" s="128"/>
+      <c r="D8" s="129"/>
       <c r="E8" s="45">
         <v>0.77083333333333337</v>
       </c>
@@ -2989,17 +2970,17 @@
       </c>
       <c r="K8" s="47"/>
       <c r="L8" s="48"/>
-      <c r="M8" s="117"/>
-      <c r="N8" s="118"/>
+      <c r="M8" s="147"/>
+      <c r="N8" s="148"/>
       <c r="O8" s="10"/>
     </row>
     <row r="9" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A9" s="2"/>
-      <c r="B9" s="138"/>
-      <c r="C9" s="142" t="s">
+      <c r="B9" s="137"/>
+      <c r="C9" s="128" t="s">
         <v>27</v>
       </c>
-      <c r="D9" s="143"/>
+      <c r="D9" s="129"/>
       <c r="E9" s="40">
         <v>0.39583333333333331</v>
       </c>
@@ -3024,17 +3005,17 @@
       <c r="L9" s="41">
         <v>0.77083333333333337</v>
       </c>
-      <c r="M9" s="125"/>
-      <c r="N9" s="126"/>
+      <c r="M9" s="145"/>
+      <c r="N9" s="146"/>
       <c r="O9" s="10"/>
     </row>
     <row r="10" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A10" s="2"/>
-      <c r="B10" s="138"/>
-      <c r="C10" s="142" t="s">
+      <c r="B10" s="137"/>
+      <c r="C10" s="128" t="s">
         <v>28</v>
       </c>
-      <c r="D10" s="143"/>
+      <c r="D10" s="129"/>
       <c r="E10" s="45">
         <v>0.36458333333333331</v>
       </c>
@@ -3051,15 +3032,15 @@
       </c>
       <c r="K10" s="47"/>
       <c r="L10" s="48"/>
-      <c r="M10" s="117"/>
-      <c r="N10" s="118"/>
+      <c r="M10" s="147"/>
+      <c r="N10" s="148"/>
       <c r="O10" s="10"/>
     </row>
     <row r="11" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A11" s="2"/>
-      <c r="B11" s="138"/>
-      <c r="C11" s="142"/>
-      <c r="D11" s="143"/>
+      <c r="B11" s="137"/>
+      <c r="C11" s="128"/>
+      <c r="D11" s="129"/>
       <c r="E11" s="40">
         <v>0.66666666666666663</v>
       </c>
@@ -3076,17 +3057,17 @@
       </c>
       <c r="K11" s="40"/>
       <c r="L11" s="41"/>
-      <c r="M11" s="125"/>
-      <c r="N11" s="126"/>
+      <c r="M11" s="145"/>
+      <c r="N11" s="146"/>
       <c r="O11" s="10"/>
     </row>
     <row r="12" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>
-      <c r="B12" s="138"/>
-      <c r="C12" s="135" t="s">
+      <c r="B12" s="137"/>
+      <c r="C12" s="134" t="s">
         <v>29</v>
       </c>
-      <c r="D12" s="136"/>
+      <c r="D12" s="135"/>
       <c r="E12" s="45">
         <v>0.33333333333333331</v>
       </c>
@@ -3103,17 +3084,17 @@
       </c>
       <c r="K12" s="45"/>
       <c r="L12" s="46"/>
-      <c r="M12" s="117" t="s">
+      <c r="M12" s="147" t="s">
         <v>36</v>
       </c>
-      <c r="N12" s="118"/>
+      <c r="N12" s="148"/>
       <c r="O12" s="10"/>
     </row>
     <row r="13" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A13" s="2"/>
-      <c r="B13" s="138"/>
-      <c r="C13" s="135"/>
-      <c r="D13" s="136"/>
+      <c r="B13" s="137"/>
+      <c r="C13" s="134"/>
+      <c r="D13" s="135"/>
       <c r="E13" s="40">
         <v>0.45833333333333331</v>
       </c>
@@ -3130,15 +3111,15 @@
       </c>
       <c r="K13" s="40"/>
       <c r="L13" s="41"/>
-      <c r="M13" s="125"/>
-      <c r="N13" s="126"/>
+      <c r="M13" s="145"/>
+      <c r="N13" s="146"/>
       <c r="O13" s="10"/>
     </row>
     <row r="14" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A14" s="2"/>
-      <c r="B14" s="138"/>
-      <c r="C14" s="135"/>
-      <c r="D14" s="136"/>
+      <c r="B14" s="137"/>
+      <c r="C14" s="134"/>
+      <c r="D14" s="135"/>
       <c r="E14" s="45"/>
       <c r="F14" s="46"/>
       <c r="G14" s="45">
@@ -3155,15 +3136,15 @@
       <c r="L14" s="46">
         <v>0.72916666666666663</v>
       </c>
-      <c r="M14" s="117"/>
-      <c r="N14" s="118"/>
+      <c r="M14" s="147"/>
+      <c r="N14" s="148"/>
       <c r="O14" s="10"/>
     </row>
     <row r="15" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A15" s="2"/>
-      <c r="B15" s="138"/>
-      <c r="C15" s="135"/>
-      <c r="D15" s="136"/>
+      <c r="B15" s="137"/>
+      <c r="C15" s="134"/>
+      <c r="D15" s="135"/>
       <c r="E15" s="40"/>
       <c r="F15" s="41"/>
       <c r="G15" s="40">
@@ -3180,19 +3161,19 @@
       <c r="L15" s="41">
         <v>0.77083333333333337</v>
       </c>
-      <c r="M15" s="125"/>
-      <c r="N15" s="126"/>
+      <c r="M15" s="145"/>
+      <c r="N15" s="146"/>
       <c r="O15" s="10"/>
     </row>
     <row r="16" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
-      <c r="B16" s="139" t="s">
+      <c r="B16" s="130" t="s">
         <v>31</v>
       </c>
-      <c r="C16" s="144" t="s">
+      <c r="C16" s="124" t="s">
         <v>27</v>
       </c>
-      <c r="D16" s="133"/>
+      <c r="D16" s="125"/>
       <c r="E16" s="8"/>
       <c r="F16" s="9"/>
       <c r="G16" s="8">
@@ -3209,15 +3190,15 @@
       <c r="L16" s="9">
         <v>0.42708333333333331</v>
       </c>
-      <c r="M16" s="123"/>
-      <c r="N16" s="124"/>
+      <c r="M16" s="153"/>
+      <c r="N16" s="154"/>
       <c r="O16" s="10"/>
     </row>
     <row r="17" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A17" s="2"/>
-      <c r="B17" s="139"/>
-      <c r="C17" s="144"/>
-      <c r="D17" s="133"/>
+      <c r="B17" s="130"/>
+      <c r="C17" s="124"/>
+      <c r="D17" s="125"/>
       <c r="E17" s="8"/>
       <c r="F17" s="9"/>
       <c r="G17" s="8">
@@ -3234,17 +3215,17 @@
       <c r="L17" s="9">
         <v>0.80208333333333337</v>
       </c>
-      <c r="M17" s="123"/>
-      <c r="N17" s="124"/>
+      <c r="M17" s="153"/>
+      <c r="N17" s="154"/>
       <c r="O17" s="10"/>
     </row>
     <row r="18" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A18" s="2"/>
-      <c r="B18" s="139"/>
-      <c r="C18" s="144" t="s">
+      <c r="B18" s="130"/>
+      <c r="C18" s="124" t="s">
         <v>28</v>
       </c>
-      <c r="D18" s="133"/>
+      <c r="D18" s="125"/>
       <c r="E18" s="8"/>
       <c r="F18" s="9"/>
       <c r="G18" s="8">
@@ -3261,15 +3242,15 @@
       <c r="L18" s="9">
         <v>0.39583333333333331</v>
       </c>
-      <c r="M18" s="123"/>
-      <c r="N18" s="124"/>
+      <c r="M18" s="153"/>
+      <c r="N18" s="154"/>
       <c r="O18" s="10"/>
     </row>
     <row r="19" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A19" s="2"/>
-      <c r="B19" s="139"/>
-      <c r="C19" s="144"/>
-      <c r="D19" s="133"/>
+      <c r="B19" s="130"/>
+      <c r="C19" s="124"/>
+      <c r="D19" s="125"/>
       <c r="E19" s="8"/>
       <c r="F19" s="9"/>
       <c r="G19" s="8">
@@ -3286,17 +3267,17 @@
       <c r="L19" s="9">
         <v>0.69791666666666663</v>
       </c>
-      <c r="M19" s="123"/>
-      <c r="N19" s="124"/>
+      <c r="M19" s="153"/>
+      <c r="N19" s="154"/>
       <c r="O19" s="10"/>
     </row>
     <row r="20" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A20" s="2"/>
-      <c r="B20" s="139"/>
-      <c r="C20" s="145" t="s">
+      <c r="B20" s="130"/>
+      <c r="C20" s="126" t="s">
         <v>29</v>
       </c>
-      <c r="D20" s="146"/>
+      <c r="D20" s="127"/>
       <c r="E20" s="8"/>
       <c r="F20" s="9"/>
       <c r="G20" s="8">
@@ -3313,17 +3294,17 @@
       <c r="L20" s="9">
         <v>0.36458333333333331</v>
       </c>
-      <c r="M20" s="123" t="s">
+      <c r="M20" s="153" t="s">
         <v>37</v>
       </c>
-      <c r="N20" s="124"/>
+      <c r="N20" s="154"/>
       <c r="O20" s="10"/>
     </row>
     <row r="21" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A21" s="2"/>
-      <c r="B21" s="139"/>
-      <c r="C21" s="145"/>
-      <c r="D21" s="146"/>
+      <c r="B21" s="130"/>
+      <c r="C21" s="126"/>
+      <c r="D21" s="127"/>
       <c r="E21" s="8"/>
       <c r="F21" s="9"/>
       <c r="G21" s="8">
@@ -3340,19 +3321,19 @@
       <c r="L21" s="9">
         <v>0.83333333333333337</v>
       </c>
-      <c r="M21" s="123"/>
-      <c r="N21" s="124"/>
+      <c r="M21" s="153"/>
+      <c r="N21" s="154"/>
       <c r="O21" s="10"/>
     </row>
     <row r="22" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A22" s="2"/>
-      <c r="B22" s="138" t="s">
+      <c r="B22" s="137" t="s">
         <v>33</v>
       </c>
-      <c r="C22" s="142" t="s">
+      <c r="C22" s="128" t="s">
         <v>28</v>
       </c>
-      <c r="D22" s="143"/>
+      <c r="D22" s="129"/>
       <c r="E22" s="45">
         <v>0.69791666666666663</v>
       </c>
@@ -3369,17 +3350,17 @@
       </c>
       <c r="K22" s="45"/>
       <c r="L22" s="46"/>
-      <c r="M22" s="117"/>
-      <c r="N22" s="118"/>
+      <c r="M22" s="147"/>
+      <c r="N22" s="148"/>
       <c r="O22" s="10"/>
     </row>
     <row r="23" spans="1:15" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2"/>
-      <c r="B23" s="138"/>
-      <c r="C23" s="142" t="s">
+      <c r="B23" s="137"/>
+      <c r="C23" s="128" t="s">
         <v>29</v>
       </c>
-      <c r="D23" s="143"/>
+      <c r="D23" s="129"/>
       <c r="E23" s="45">
         <v>0.80208333333333337</v>
       </c>
@@ -3396,52 +3377,52 @@
       </c>
       <c r="K23" s="45"/>
       <c r="L23" s="46"/>
-      <c r="M23" s="117"/>
-      <c r="N23" s="118"/>
+      <c r="M23" s="147"/>
+      <c r="N23" s="148"/>
       <c r="O23" s="10"/>
     </row>
     <row r="24" spans="1:15" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2"/>
-      <c r="B24" s="139" t="s">
+      <c r="B24" s="130" t="s">
         <v>30</v>
       </c>
-      <c r="C24" s="145"/>
-      <c r="D24" s="146"/>
-      <c r="E24" s="127">
+      <c r="C24" s="126"/>
+      <c r="D24" s="127"/>
+      <c r="E24" s="138">
         <v>0.5</v>
       </c>
-      <c r="F24" s="129">
+      <c r="F24" s="122">
         <v>0.53125</v>
       </c>
-      <c r="G24" s="127"/>
-      <c r="H24" s="129"/>
-      <c r="I24" s="131">
+      <c r="G24" s="138"/>
+      <c r="H24" s="122"/>
+      <c r="I24" s="142">
         <v>0.5</v>
       </c>
-      <c r="J24" s="133">
+      <c r="J24" s="125">
         <v>0.53125</v>
       </c>
-      <c r="K24" s="127"/>
-      <c r="L24" s="133"/>
-      <c r="M24" s="119"/>
-      <c r="N24" s="120"/>
+      <c r="K24" s="138"/>
+      <c r="L24" s="125"/>
+      <c r="M24" s="149"/>
+      <c r="N24" s="150"/>
       <c r="O24" s="10"/>
     </row>
     <row r="25" spans="1:15" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="2"/>
-      <c r="B25" s="147"/>
-      <c r="C25" s="148"/>
-      <c r="D25" s="149"/>
-      <c r="E25" s="128"/>
-      <c r="F25" s="130"/>
-      <c r="G25" s="128"/>
-      <c r="H25" s="130"/>
-      <c r="I25" s="132"/>
-      <c r="J25" s="134"/>
-      <c r="K25" s="128"/>
-      <c r="L25" s="134"/>
-      <c r="M25" s="121"/>
-      <c r="N25" s="122"/>
+      <c r="B25" s="131"/>
+      <c r="C25" s="132"/>
+      <c r="D25" s="133"/>
+      <c r="E25" s="139"/>
+      <c r="F25" s="123"/>
+      <c r="G25" s="139"/>
+      <c r="H25" s="123"/>
+      <c r="I25" s="143"/>
+      <c r="J25" s="144"/>
+      <c r="K25" s="139"/>
+      <c r="L25" s="144"/>
+      <c r="M25" s="151"/>
+      <c r="N25" s="152"/>
       <c r="O25" s="10"/>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
@@ -3482,35 +3463,15 @@
     </row>
   </sheetData>
   <mergeCells count="49">
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="E4:F4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="M4:N4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="K4:L4"/>
-    <mergeCell ref="F24:F25"/>
-    <mergeCell ref="C16:D17"/>
-    <mergeCell ref="C18:D19"/>
-    <mergeCell ref="C20:D21"/>
-    <mergeCell ref="C22:D22"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="B24:D25"/>
-    <mergeCell ref="C12:D15"/>
-    <mergeCell ref="B5:B15"/>
-    <mergeCell ref="B16:B21"/>
-    <mergeCell ref="B22:B23"/>
-    <mergeCell ref="E24:E25"/>
-    <mergeCell ref="C5:D6"/>
-    <mergeCell ref="C7:D8"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="C10:D11"/>
-    <mergeCell ref="G24:G25"/>
-    <mergeCell ref="H24:H25"/>
-    <mergeCell ref="I24:I25"/>
-    <mergeCell ref="L24:L25"/>
-    <mergeCell ref="J24:J25"/>
-    <mergeCell ref="K24:K25"/>
+    <mergeCell ref="M22:N22"/>
+    <mergeCell ref="M23:N23"/>
+    <mergeCell ref="M24:N25"/>
+    <mergeCell ref="M16:N16"/>
+    <mergeCell ref="M17:N17"/>
+    <mergeCell ref="M18:N18"/>
+    <mergeCell ref="M19:N19"/>
+    <mergeCell ref="M20:N20"/>
+    <mergeCell ref="M21:N21"/>
     <mergeCell ref="M15:N15"/>
     <mergeCell ref="M5:N5"/>
     <mergeCell ref="M6:N6"/>
@@ -3522,15 +3483,35 @@
     <mergeCell ref="M12:N12"/>
     <mergeCell ref="M13:N13"/>
     <mergeCell ref="M14:N14"/>
-    <mergeCell ref="M22:N22"/>
-    <mergeCell ref="M23:N23"/>
-    <mergeCell ref="M24:N25"/>
-    <mergeCell ref="M16:N16"/>
-    <mergeCell ref="M17:N17"/>
-    <mergeCell ref="M18:N18"/>
-    <mergeCell ref="M19:N19"/>
-    <mergeCell ref="M20:N20"/>
-    <mergeCell ref="M21:N21"/>
+    <mergeCell ref="G24:G25"/>
+    <mergeCell ref="H24:H25"/>
+    <mergeCell ref="I24:I25"/>
+    <mergeCell ref="L24:L25"/>
+    <mergeCell ref="J24:J25"/>
+    <mergeCell ref="K24:K25"/>
+    <mergeCell ref="C12:D15"/>
+    <mergeCell ref="B5:B15"/>
+    <mergeCell ref="B16:B21"/>
+    <mergeCell ref="B22:B23"/>
+    <mergeCell ref="E24:E25"/>
+    <mergeCell ref="C5:D6"/>
+    <mergeCell ref="C7:D8"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="C10:D11"/>
+    <mergeCell ref="F24:F25"/>
+    <mergeCell ref="C16:D17"/>
+    <mergeCell ref="C18:D19"/>
+    <mergeCell ref="C20:D21"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="B24:D25"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="K4:L4"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
@@ -3603,23 +3584,23 @@
       <c r="D3" s="157" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="152"/>
-      <c r="F3" s="151" t="s">
+      <c r="E3" s="119"/>
+      <c r="F3" s="118" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="152"/>
-      <c r="H3" s="151" t="s">
+      <c r="G3" s="119"/>
+      <c r="H3" s="118" t="s">
         <v>4</v>
       </c>
-      <c r="I3" s="152"/>
-      <c r="J3" s="151" t="s">
+      <c r="I3" s="119"/>
+      <c r="J3" s="118" t="s">
         <v>5</v>
       </c>
-      <c r="K3" s="152"/>
-      <c r="L3" s="151" t="s">
+      <c r="K3" s="119"/>
+      <c r="L3" s="118" t="s">
         <v>6</v>
       </c>
-      <c r="M3" s="152"/>
+      <c r="M3" s="119"/>
       <c r="N3" s="2"/>
     </row>
     <row r="4" spans="1:14" ht="18.75" x14ac:dyDescent="0.25">
@@ -4134,10 +4115,10 @@
       <c r="E4" s="65" t="s">
         <v>68</v>
       </c>
-      <c r="F4" s="179" t="s">
+      <c r="F4" s="170" t="s">
         <v>69</v>
       </c>
-      <c r="G4" s="179"/>
+      <c r="G4" s="170"/>
       <c r="H4" s="66" t="s">
         <v>73</v>
       </c>
@@ -4148,10 +4129,10 @@
     </row>
     <row r="5" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A5" s="2"/>
-      <c r="B5" s="164" t="s">
+      <c r="B5" s="189" t="s">
         <v>66</v>
       </c>
-      <c r="C5" s="131" t="s">
+      <c r="C5" s="142" t="s">
         <v>40</v>
       </c>
       <c r="D5" s="16" t="s">
@@ -4166,18 +4147,18 @@
       <c r="G5" s="16">
         <v>0.39583333333333331</v>
       </c>
-      <c r="H5" s="187">
+      <c r="H5" s="178">
         <v>10</v>
       </c>
-      <c r="I5" s="133" t="s">
+      <c r="I5" s="125" t="s">
         <v>90</v>
       </c>
       <c r="J5" s="2"/>
     </row>
     <row r="6" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2"/>
-      <c r="B6" s="164"/>
-      <c r="C6" s="132"/>
+      <c r="B6" s="189"/>
+      <c r="C6" s="143"/>
       <c r="D6" s="67" t="s">
         <v>46</v>
       </c>
@@ -4190,14 +4171,14 @@
       <c r="G6" s="67">
         <v>0.75</v>
       </c>
-      <c r="H6" s="188"/>
-      <c r="I6" s="134"/>
+      <c r="H6" s="179"/>
+      <c r="I6" s="144"/>
       <c r="J6" s="2"/>
     </row>
     <row r="7" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
-      <c r="B7" s="164"/>
-      <c r="C7" s="166" t="s">
+      <c r="B7" s="189"/>
+      <c r="C7" s="191" t="s">
         <v>43</v>
       </c>
       <c r="D7" s="72" t="s">
@@ -4212,18 +4193,18 @@
       <c r="G7" s="69">
         <v>0.41666666666666669</v>
       </c>
-      <c r="H7" s="183">
+      <c r="H7" s="174">
         <v>16</v>
       </c>
-      <c r="I7" s="180" t="s">
+      <c r="I7" s="171" t="s">
         <v>91</v>
       </c>
       <c r="J7" s="2"/>
     </row>
     <row r="8" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A8" s="2"/>
-      <c r="B8" s="164"/>
-      <c r="C8" s="167"/>
+      <c r="B8" s="189"/>
+      <c r="C8" s="192"/>
       <c r="D8" s="23" t="s">
         <v>48</v>
       </c>
@@ -4236,14 +4217,14 @@
       <c r="G8" s="60">
         <v>0.76041666666666663</v>
       </c>
-      <c r="H8" s="184"/>
-      <c r="I8" s="176"/>
+      <c r="H8" s="175"/>
+      <c r="I8" s="167"/>
       <c r="J8" s="10"/>
     </row>
     <row r="9" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A9" s="2"/>
-      <c r="B9" s="164"/>
-      <c r="C9" s="167"/>
+      <c r="B9" s="189"/>
+      <c r="C9" s="192"/>
       <c r="D9" s="23" t="s">
         <v>49</v>
       </c>
@@ -4256,28 +4237,28 @@
       <c r="G9" s="60">
         <v>0.79166666666666663</v>
       </c>
-      <c r="H9" s="184"/>
-      <c r="I9" s="176" t="s">
+      <c r="H9" s="175"/>
+      <c r="I9" s="167" t="s">
         <v>92</v>
       </c>
       <c r="J9" s="10"/>
     </row>
     <row r="10" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2"/>
-      <c r="B10" s="164"/>
-      <c r="C10" s="168"/>
+      <c r="B10" s="189"/>
+      <c r="C10" s="193"/>
       <c r="D10" s="30"/>
       <c r="E10" s="71"/>
       <c r="F10" s="71"/>
       <c r="G10" s="71"/>
-      <c r="H10" s="185"/>
-      <c r="I10" s="177"/>
+      <c r="H10" s="176"/>
+      <c r="I10" s="168"/>
       <c r="J10" s="10"/>
     </row>
     <row r="11" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A11" s="2"/>
-      <c r="B11" s="164"/>
-      <c r="C11" s="169" t="s">
+      <c r="B11" s="189"/>
+      <c r="C11" s="194" t="s">
         <v>71</v>
       </c>
       <c r="D11" s="75" t="s">
@@ -4292,7 +4273,7 @@
       <c r="G11" s="76">
         <v>0.45833333333333331</v>
       </c>
-      <c r="H11" s="189">
+      <c r="H11" s="180">
         <v>14</v>
       </c>
       <c r="I11" s="77" t="s">
@@ -4302,8 +4283,8 @@
     </row>
     <row r="12" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>
-      <c r="B12" s="164"/>
-      <c r="C12" s="170"/>
+      <c r="B12" s="189"/>
+      <c r="C12" s="195"/>
       <c r="D12" s="78" t="s">
         <v>74</v>
       </c>
@@ -4316,7 +4297,7 @@
       <c r="G12" s="61">
         <v>0.45833333333333331</v>
       </c>
-      <c r="H12" s="190"/>
+      <c r="H12" s="181"/>
       <c r="I12" s="57" t="s">
         <v>91</v>
       </c>
@@ -4324,8 +4305,8 @@
     </row>
     <row r="13" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A13" s="2"/>
-      <c r="B13" s="164"/>
-      <c r="C13" s="170"/>
+      <c r="B13" s="189"/>
+      <c r="C13" s="195"/>
       <c r="D13" s="78" t="s">
         <v>74</v>
       </c>
@@ -4338,16 +4319,16 @@
       <c r="G13" s="61">
         <v>0.77083333333333337</v>
       </c>
-      <c r="H13" s="190"/>
-      <c r="I13" s="181" t="s">
+      <c r="H13" s="181"/>
+      <c r="I13" s="172" t="s">
         <v>93</v>
       </c>
       <c r="J13" s="10"/>
     </row>
     <row r="14" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A14" s="2"/>
-      <c r="B14" s="164"/>
-      <c r="C14" s="170"/>
+      <c r="B14" s="189"/>
+      <c r="C14" s="195"/>
       <c r="D14" s="78" t="s">
         <v>75</v>
       </c>
@@ -4360,14 +4341,14 @@
       <c r="G14" s="61">
         <v>0.45833333333333331</v>
       </c>
-      <c r="H14" s="190"/>
-      <c r="I14" s="181"/>
+      <c r="H14" s="181"/>
+      <c r="I14" s="172"/>
       <c r="J14" s="10"/>
     </row>
     <row r="15" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A15" s="2"/>
-      <c r="B15" s="164"/>
-      <c r="C15" s="170"/>
+      <c r="B15" s="189"/>
+      <c r="C15" s="195"/>
       <c r="D15" s="78" t="s">
         <v>75</v>
       </c>
@@ -4380,14 +4361,14 @@
       <c r="G15" s="61">
         <v>0.80208333333333337</v>
       </c>
-      <c r="H15" s="190"/>
-      <c r="I15" s="181"/>
+      <c r="H15" s="181"/>
+      <c r="I15" s="172"/>
       <c r="J15" s="10"/>
     </row>
     <row r="16" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
-      <c r="B16" s="164"/>
-      <c r="C16" s="170"/>
+      <c r="B16" s="189"/>
+      <c r="C16" s="195"/>
       <c r="D16" s="78" t="s">
         <v>76</v>
       </c>
@@ -4400,14 +4381,14 @@
       <c r="G16" s="61">
         <v>0.42708333333333331</v>
       </c>
-      <c r="H16" s="190"/>
-      <c r="I16" s="181"/>
+      <c r="H16" s="181"/>
+      <c r="I16" s="172"/>
       <c r="J16" s="10"/>
     </row>
     <row r="17" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A17" s="2"/>
-      <c r="B17" s="164"/>
-      <c r="C17" s="170"/>
+      <c r="B17" s="189"/>
+      <c r="C17" s="195"/>
       <c r="D17" s="78" t="s">
         <v>76</v>
       </c>
@@ -4420,14 +4401,14 @@
       <c r="G17" s="61">
         <v>0.77083333333333337</v>
       </c>
-      <c r="H17" s="190"/>
-      <c r="I17" s="181"/>
+      <c r="H17" s="181"/>
+      <c r="I17" s="172"/>
       <c r="J17" s="10"/>
     </row>
     <row r="18" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A18" s="2"/>
-      <c r="B18" s="164"/>
-      <c r="C18" s="170"/>
+      <c r="B18" s="189"/>
+      <c r="C18" s="195"/>
       <c r="D18" s="78" t="s">
         <v>77</v>
       </c>
@@ -4440,14 +4421,14 @@
       <c r="G18" s="61">
         <v>0.39583333333333331</v>
       </c>
-      <c r="H18" s="190"/>
-      <c r="I18" s="181"/>
+      <c r="H18" s="181"/>
+      <c r="I18" s="172"/>
       <c r="J18" s="10"/>
     </row>
     <row r="19" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2"/>
-      <c r="B19" s="164"/>
-      <c r="C19" s="170"/>
+      <c r="B19" s="189"/>
+      <c r="C19" s="195"/>
       <c r="D19" s="79" t="s">
         <v>77</v>
       </c>
@@ -4460,14 +4441,14 @@
       <c r="G19" s="80">
         <v>0.69791666666666663</v>
       </c>
-      <c r="H19" s="191"/>
-      <c r="I19" s="182"/>
+      <c r="H19" s="182"/>
+      <c r="I19" s="173"/>
       <c r="J19" s="10"/>
     </row>
     <row r="20" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A20" s="2"/>
-      <c r="B20" s="164"/>
-      <c r="C20" s="170"/>
+      <c r="B20" s="189"/>
+      <c r="C20" s="195"/>
       <c r="D20" s="81" t="s">
         <v>78</v>
       </c>
@@ -4480,7 +4461,7 @@
       <c r="G20" s="82">
         <v>0.36458333333333331</v>
       </c>
-      <c r="H20" s="192">
+      <c r="H20" s="183">
         <v>12</v>
       </c>
       <c r="I20" s="83" t="s">
@@ -4490,8 +4471,8 @@
     </row>
     <row r="21" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A21" s="2"/>
-      <c r="B21" s="164"/>
-      <c r="C21" s="170"/>
+      <c r="B21" s="189"/>
+      <c r="C21" s="195"/>
       <c r="D21" s="84" t="s">
         <v>78</v>
       </c>
@@ -4504,7 +4485,7 @@
       <c r="G21" s="62">
         <v>0.48958333333333331</v>
       </c>
-      <c r="H21" s="193"/>
+      <c r="H21" s="184"/>
       <c r="I21" s="58" t="s">
         <v>94</v>
       </c>
@@ -4512,8 +4493,8 @@
     </row>
     <row r="22" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A22" s="2"/>
-      <c r="B22" s="164"/>
-      <c r="C22" s="170"/>
+      <c r="B22" s="189"/>
+      <c r="C22" s="195"/>
       <c r="D22" s="84" t="s">
         <v>78</v>
       </c>
@@ -4526,7 +4507,7 @@
       <c r="G22" s="62">
         <v>0.72916666666666663</v>
       </c>
-      <c r="H22" s="193"/>
+      <c r="H22" s="184"/>
       <c r="I22" s="58" t="s">
         <v>93</v>
       </c>
@@ -4534,8 +4515,8 @@
     </row>
     <row r="23" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A23" s="2"/>
-      <c r="B23" s="164"/>
-      <c r="C23" s="170"/>
+      <c r="B23" s="189"/>
+      <c r="C23" s="195"/>
       <c r="D23" s="84" t="s">
         <v>78</v>
       </c>
@@ -4548,7 +4529,7 @@
       <c r="G23" s="62">
         <v>0.77083333333333337</v>
       </c>
-      <c r="H23" s="193"/>
+      <c r="H23" s="184"/>
       <c r="I23" s="58" t="s">
         <v>92</v>
       </c>
@@ -4556,8 +4537,8 @@
     </row>
     <row r="24" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="2"/>
-      <c r="B24" s="164"/>
-      <c r="C24" s="170"/>
+      <c r="B24" s="189"/>
+      <c r="C24" s="195"/>
       <c r="D24" s="85" t="s">
         <v>78</v>
       </c>
@@ -4570,7 +4551,7 @@
       <c r="G24" s="86">
         <v>0.46875</v>
       </c>
-      <c r="H24" s="194"/>
+      <c r="H24" s="185"/>
       <c r="I24" s="87" t="s">
         <v>94</v>
       </c>
@@ -4578,8 +4559,8 @@
     </row>
     <row r="25" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A25" s="2"/>
-      <c r="B25" s="164"/>
-      <c r="C25" s="170"/>
+      <c r="B25" s="189"/>
+      <c r="C25" s="195"/>
       <c r="D25" s="88" t="s">
         <v>79</v>
       </c>
@@ -4592,18 +4573,18 @@
       <c r="G25" s="89">
         <v>0.42708333333333331</v>
       </c>
-      <c r="H25" s="195">
+      <c r="H25" s="186">
         <v>14</v>
       </c>
-      <c r="I25" s="173" t="s">
+      <c r="I25" s="164" t="s">
         <v>93</v>
       </c>
       <c r="J25" s="10"/>
     </row>
     <row r="26" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A26" s="2"/>
-      <c r="B26" s="164"/>
-      <c r="C26" s="170"/>
+      <c r="B26" s="189"/>
+      <c r="C26" s="195"/>
       <c r="D26" s="90" t="s">
         <v>79</v>
       </c>
@@ -4616,14 +4597,14 @@
       <c r="G26" s="63">
         <v>0.80208333333333337</v>
       </c>
-      <c r="H26" s="196"/>
-      <c r="I26" s="174"/>
+      <c r="H26" s="187"/>
+      <c r="I26" s="165"/>
       <c r="J26" s="10"/>
     </row>
     <row r="27" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A27" s="2"/>
-      <c r="B27" s="164"/>
-      <c r="C27" s="170"/>
+      <c r="B27" s="189"/>
+      <c r="C27" s="195"/>
       <c r="D27" s="90" t="s">
         <v>80</v>
       </c>
@@ -4636,14 +4617,14 @@
       <c r="G27" s="63">
         <v>0.39583333333333331</v>
       </c>
-      <c r="H27" s="196"/>
-      <c r="I27" s="174"/>
+      <c r="H27" s="187"/>
+      <c r="I27" s="165"/>
       <c r="J27" s="10"/>
     </row>
     <row r="28" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="2"/>
-      <c r="B28" s="164"/>
-      <c r="C28" s="170"/>
+      <c r="B28" s="189"/>
+      <c r="C28" s="195"/>
       <c r="D28" s="91" t="s">
         <v>80</v>
       </c>
@@ -4656,14 +4637,14 @@
       <c r="G28" s="92">
         <v>0.69791666666666663</v>
       </c>
-      <c r="H28" s="197"/>
-      <c r="I28" s="175"/>
+      <c r="H28" s="188"/>
+      <c r="I28" s="166"/>
       <c r="J28" s="10"/>
     </row>
     <row r="29" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A29" s="2"/>
-      <c r="B29" s="164"/>
-      <c r="C29" s="170"/>
+      <c r="B29" s="189"/>
+      <c r="C29" s="195"/>
       <c r="D29" s="93" t="s">
         <v>81</v>
       </c>
@@ -4676,7 +4657,7 @@
       <c r="G29" s="69">
         <v>0.36458333333333331</v>
       </c>
-      <c r="H29" s="183">
+      <c r="H29" s="174">
         <v>12</v>
       </c>
       <c r="I29" s="94" t="s">
@@ -4686,8 +4667,8 @@
     </row>
     <row r="30" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A30" s="2"/>
-      <c r="B30" s="164"/>
-      <c r="C30" s="170"/>
+      <c r="B30" s="189"/>
+      <c r="C30" s="195"/>
       <c r="D30" s="25" t="s">
         <v>81</v>
       </c>
@@ -4700,16 +4681,16 @@
       <c r="G30" s="60">
         <v>0.83333333333333337</v>
       </c>
-      <c r="H30" s="184"/>
-      <c r="I30" s="176" t="s">
+      <c r="H30" s="175"/>
+      <c r="I30" s="167" t="s">
         <v>94</v>
       </c>
       <c r="J30" s="10"/>
     </row>
     <row r="31" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="2"/>
-      <c r="B31" s="164"/>
-      <c r="C31" s="170"/>
+      <c r="B31" s="189"/>
+      <c r="C31" s="195"/>
       <c r="D31" s="33" t="s">
         <v>81</v>
       </c>
@@ -4722,14 +4703,14 @@
       <c r="G31" s="70">
         <v>0.41666666666666669</v>
       </c>
-      <c r="H31" s="185"/>
-      <c r="I31" s="177"/>
+      <c r="H31" s="176"/>
+      <c r="I31" s="168"/>
       <c r="J31" s="10"/>
     </row>
     <row r="32" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A32" s="2"/>
-      <c r="B32" s="164"/>
-      <c r="C32" s="170"/>
+      <c r="B32" s="189"/>
+      <c r="C32" s="195"/>
       <c r="D32" s="75" t="s">
         <v>83</v>
       </c>
@@ -4752,8 +4733,8 @@
     </row>
     <row r="33" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A33" s="2"/>
-      <c r="B33" s="164"/>
-      <c r="C33" s="170"/>
+      <c r="B33" s="189"/>
+      <c r="C33" s="195"/>
       <c r="D33" s="84" t="s">
         <v>84</v>
       </c>
@@ -4776,8 +4757,8 @@
     </row>
     <row r="34" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="2"/>
-      <c r="B34" s="164"/>
-      <c r="C34" s="171"/>
+      <c r="B34" s="189"/>
+      <c r="C34" s="196"/>
       <c r="D34" s="79" t="s">
         <v>82</v>
       </c>
@@ -4800,8 +4781,8 @@
     </row>
     <row r="35" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A35" s="2"/>
-      <c r="B35" s="164"/>
-      <c r="C35" s="172" t="s">
+      <c r="B35" s="189"/>
+      <c r="C35" s="197" t="s">
         <v>44</v>
       </c>
       <c r="D35" s="99" t="s">
@@ -4816,7 +4797,7 @@
       <c r="G35" s="69">
         <v>0.77083333333333337</v>
       </c>
-      <c r="H35" s="183">
+      <c r="H35" s="174">
         <v>20</v>
       </c>
       <c r="I35" s="100" t="s">
@@ -4826,7 +4807,7 @@
     </row>
     <row r="36" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A36" s="2"/>
-      <c r="B36" s="164"/>
+      <c r="B36" s="189"/>
       <c r="C36" s="155"/>
       <c r="D36" s="27" t="s">
         <v>48</v>
@@ -4840,7 +4821,7 @@
       <c r="G36" s="60">
         <v>0.78472222222222221</v>
       </c>
-      <c r="H36" s="184"/>
+      <c r="H36" s="175"/>
       <c r="I36" s="24" t="s">
         <v>94</v>
       </c>
@@ -4848,7 +4829,7 @@
     </row>
     <row r="37" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A37" s="2"/>
-      <c r="B37" s="164"/>
+      <c r="B37" s="189"/>
       <c r="C37" s="155"/>
       <c r="D37" s="27" t="s">
         <v>49</v>
@@ -4862,7 +4843,7 @@
       <c r="G37" s="60">
         <v>0.80555555555555558</v>
       </c>
-      <c r="H37" s="184"/>
+      <c r="H37" s="175"/>
       <c r="I37" s="24" t="s">
         <v>91</v>
       </c>
@@ -4870,7 +4851,7 @@
     </row>
     <row r="38" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A38" s="2"/>
-      <c r="B38" s="164"/>
+      <c r="B38" s="189"/>
       <c r="C38" s="155"/>
       <c r="D38" s="27" t="s">
         <v>49</v>
@@ -4884,7 +4865,7 @@
       <c r="G38" s="60">
         <v>0.81944444444444442</v>
       </c>
-      <c r="H38" s="184"/>
+      <c r="H38" s="175"/>
       <c r="I38" s="24" t="s">
         <v>94</v>
       </c>
@@ -4892,7 +4873,7 @@
     </row>
     <row r="39" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A39" s="2"/>
-      <c r="B39" s="164"/>
+      <c r="B39" s="189"/>
       <c r="C39" s="155"/>
       <c r="D39" s="27" t="s">
         <v>50</v>
@@ -4906,7 +4887,7 @@
       <c r="G39" s="60">
         <v>0.84027777777777779</v>
       </c>
-      <c r="H39" s="184"/>
+      <c r="H39" s="175"/>
       <c r="I39" s="24" t="s">
         <v>91</v>
       </c>
@@ -4914,7 +4895,7 @@
     </row>
     <row r="40" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A40" s="2"/>
-      <c r="B40" s="164"/>
+      <c r="B40" s="189"/>
       <c r="C40" s="155"/>
       <c r="D40" s="27" t="s">
         <v>50</v>
@@ -4928,7 +4909,7 @@
       <c r="G40" s="60">
         <v>0.85416666666666663</v>
       </c>
-      <c r="H40" s="184"/>
+      <c r="H40" s="175"/>
       <c r="I40" s="24" t="s">
         <v>94</v>
       </c>
@@ -4936,7 +4917,7 @@
     </row>
     <row r="41" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="2"/>
-      <c r="B41" s="164"/>
+      <c r="B41" s="189"/>
       <c r="C41" s="156"/>
       <c r="D41" s="32" t="s">
         <v>51</v>
@@ -4950,7 +4931,7 @@
       <c r="G41" s="70">
         <v>0.72222222222222221</v>
       </c>
-      <c r="H41" s="185"/>
+      <c r="H41" s="176"/>
       <c r="I41" s="31" t="s">
         <v>91</v>
       </c>
@@ -4958,8 +4939,8 @@
     </row>
     <row r="42" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A42" s="2"/>
-      <c r="B42" s="164"/>
-      <c r="C42" s="169" t="s">
+      <c r="B42" s="189"/>
+      <c r="C42" s="194" t="s">
         <v>72</v>
       </c>
       <c r="D42" s="101" t="s">
@@ -4974,18 +4955,18 @@
       <c r="G42" s="102">
         <v>0.44444444444444442</v>
       </c>
-      <c r="H42" s="186">
+      <c r="H42" s="177">
         <v>12</v>
       </c>
-      <c r="I42" s="178" t="s">
+      <c r="I42" s="169" t="s">
         <v>94</v>
       </c>
       <c r="J42" s="10"/>
     </row>
     <row r="43" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A43" s="2"/>
-      <c r="B43" s="164"/>
-      <c r="C43" s="170"/>
+      <c r="B43" s="189"/>
+      <c r="C43" s="195"/>
       <c r="D43" s="15" t="s">
         <v>48</v>
       </c>
@@ -4998,14 +4979,14 @@
       <c r="G43" s="16">
         <v>0.44444444444444442</v>
       </c>
-      <c r="H43" s="187"/>
-      <c r="I43" s="133"/>
+      <c r="H43" s="178"/>
+      <c r="I43" s="125"/>
       <c r="J43" s="10"/>
     </row>
     <row r="44" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A44" s="2"/>
-      <c r="B44" s="164"/>
-      <c r="C44" s="170"/>
+      <c r="B44" s="189"/>
+      <c r="C44" s="195"/>
       <c r="D44" s="15" t="s">
         <v>49</v>
       </c>
@@ -5018,14 +4999,14 @@
       <c r="G44" s="16">
         <v>0.40972222222222221</v>
       </c>
-      <c r="H44" s="187"/>
-      <c r="I44" s="133"/>
+      <c r="H44" s="178"/>
+      <c r="I44" s="125"/>
       <c r="J44" s="10"/>
     </row>
     <row r="45" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="2"/>
-      <c r="B45" s="164"/>
-      <c r="C45" s="171"/>
+      <c r="B45" s="189"/>
+      <c r="C45" s="196"/>
       <c r="D45" s="17" t="s">
         <v>49</v>
       </c>
@@ -5038,13 +5019,13 @@
       <c r="G45" s="67">
         <v>0.70138888888888884</v>
       </c>
-      <c r="H45" s="188"/>
-      <c r="I45" s="134"/>
+      <c r="H45" s="179"/>
+      <c r="I45" s="144"/>
       <c r="J45" s="10"/>
     </row>
     <row r="46" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="2"/>
-      <c r="B46" s="164"/>
+      <c r="B46" s="189"/>
       <c r="C46" s="73" t="s">
         <v>42</v>
       </c>
@@ -5070,7 +5051,7 @@
     </row>
     <row r="47" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="2"/>
-      <c r="B47" s="165"/>
+      <c r="B47" s="190"/>
       <c r="C47" s="74" t="s">
         <v>41</v>
       </c>
@@ -5108,6 +5089,12 @@
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="B5:B47"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="C7:C10"/>
+    <mergeCell ref="C11:C34"/>
+    <mergeCell ref="C35:C41"/>
+    <mergeCell ref="C42:C45"/>
     <mergeCell ref="I25:I28"/>
     <mergeCell ref="I30:I31"/>
     <mergeCell ref="I42:I45"/>
@@ -5124,12 +5111,6 @@
     <mergeCell ref="H20:H24"/>
     <mergeCell ref="H25:H28"/>
     <mergeCell ref="H29:H31"/>
-    <mergeCell ref="B5:B47"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="C7:C10"/>
-    <mergeCell ref="C11:C34"/>
-    <mergeCell ref="C35:C41"/>
-    <mergeCell ref="C42:C45"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
@@ -5171,7 +5152,7 @@
     <row r="2" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="str">
         <f ca="1">CHOOSE(WEEKDAY(TODAY(),2),"SEG","TER","QUA","QUI","SEX","SAB","DOM")</f>
-        <v>SEX</v>
+        <v>DOM</v>
       </c>
       <c r="B2" s="112">
         <v>0.45833333333333331</v>
@@ -5180,7 +5161,7 @@
         <v>0.90625</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>95</v>
@@ -5192,7 +5173,7 @@
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="str">
         <f ca="1">CHOOSE(WEEKDAY(TODAY(),2),"SEG","TER","QUA","QUI","SEX","SAB","DOM")</f>
-        <v>SEX</v>
+        <v>DOM</v>
       </c>
       <c r="B3" s="112">
         <v>0.45833333333333331</v>
@@ -5201,7 +5182,7 @@
         <v>0.90625</v>
       </c>
       <c r="D3" s="110" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="E3" s="110" t="s">
         <v>102</v>
@@ -5213,7 +5194,7 @@
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="str">
         <f t="shared" ref="A4:A11" ca="1" si="0">CHOOSE(WEEKDAY(TODAY(),2),"SEG","TER","QUA","QUI","SEX","SAB","DOM")</f>
-        <v>SEX</v>
+        <v>DOM</v>
       </c>
       <c r="B4" s="112">
         <v>0.45833333333333331</v>
@@ -5222,19 +5203,19 @@
         <v>0.90625</v>
       </c>
       <c r="D4" s="110" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="E4" s="110" t="s">
         <v>103</v>
       </c>
       <c r="F4" s="110" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>SEX</v>
+        <v>DOM</v>
       </c>
       <c r="B5" s="112">
         <v>0.45833333333333331</v>
@@ -5243,19 +5224,19 @@
         <v>0.90625</v>
       </c>
       <c r="D5" s="110" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="E5" s="110" t="s">
         <v>104</v>
       </c>
       <c r="F5" s="110" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>SEX</v>
+        <v>DOM</v>
       </c>
       <c r="B6" s="112">
         <v>0.45833333333333331</v>
@@ -5264,28 +5245,28 @@
         <v>0.90625</v>
       </c>
       <c r="D6" s="110" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="E6" s="110" t="s">
         <v>103</v>
       </c>
       <c r="F6" s="110" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="str">
         <f ca="1">CHOOSE(WEEKDAY(TODAY(),2),"SEG","TER","QUA","QUI","SEX","SAB","DOM")</f>
-        <v>SEX</v>
+        <v>DOM</v>
       </c>
       <c r="B7" s="112">
-        <v>0.5</v>
+        <v>0.54166666666666663</v>
       </c>
       <c r="C7" s="112">
         <v>0.90625</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>95</v>
@@ -5297,16 +5278,16 @@
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="str">
         <f ca="1">CHOOSE(WEEKDAY(TODAY(),2),"SEG","TER","QUA","QUI","SEX","SAB","DOM")</f>
-        <v>SEX</v>
+        <v>DOM</v>
       </c>
       <c r="B8" s="112">
-        <v>0.5</v>
+        <v>0.54166666666666663</v>
       </c>
       <c r="C8" s="112">
         <v>0.90625</v>
       </c>
       <c r="D8" s="110" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="E8" s="110" t="s">
         <v>102</v>
@@ -5318,79 +5299,79 @@
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>SEX</v>
+        <v>DOM</v>
       </c>
       <c r="B9" s="112">
-        <v>0.5</v>
+        <v>0.54166666666666663</v>
       </c>
       <c r="C9" s="112">
         <v>0.90625</v>
       </c>
       <c r="D9" s="110" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="E9" s="110" t="s">
         <v>103</v>
       </c>
       <c r="F9" s="110" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>SEX</v>
+        <v>DOM</v>
       </c>
       <c r="B10" s="112">
-        <v>0.5</v>
+        <v>0.54166666666666663</v>
       </c>
       <c r="C10" s="112">
         <v>0.90625</v>
       </c>
       <c r="D10" s="110" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="E10" s="110" t="s">
         <v>104</v>
       </c>
       <c r="F10" s="110" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>SEX</v>
+        <v>DOM</v>
       </c>
       <c r="B11" s="112">
-        <v>0.5</v>
+        <v>0.54166666666666663</v>
       </c>
       <c r="C11" s="112">
         <v>0.90625</v>
       </c>
       <c r="D11" s="110" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="E11" s="110" t="s">
         <v>103</v>
       </c>
       <c r="F11" s="110" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="str">
         <f ca="1">CHOOSE(WEEKDAY(TODAY(),2),"SEG","TER","QUA","QUI","SEX","SAB","DOM")</f>
-        <v>SEX</v>
+        <v>DOM</v>
       </c>
       <c r="B12" s="112">
-        <v>0.91666666666666663</v>
+        <v>0.58333333333333304</v>
       </c>
       <c r="C12" s="112">
-        <v>0.95833333333333337</v>
+        <v>0.90625</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>95</v>
@@ -5402,16 +5383,16 @@
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="str">
         <f ca="1">CHOOSE(WEEKDAY(TODAY(),2),"SEG","TER","QUA","QUI","SEX","SAB","DOM")</f>
-        <v>SEX</v>
+        <v>DOM</v>
       </c>
       <c r="B13" s="112">
-        <v>3.4722222222222224E-2</v>
+        <v>0.58333333333333304</v>
       </c>
       <c r="C13" s="112">
-        <v>7.6388888888888895E-2</v>
+        <v>0.90625</v>
       </c>
       <c r="D13" s="110" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="E13" s="110" t="s">
         <v>102</v>
@@ -5422,80 +5403,80 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="str">
-        <f t="shared" ref="A14:A25" ca="1" si="1">CHOOSE(WEEKDAY(TODAY(),2),"SEG","TER","QUA","QUI","SEX","SAB","DOM")</f>
-        <v>SEX</v>
+        <f t="shared" ref="A14:A27" ca="1" si="1">CHOOSE(WEEKDAY(TODAY(),2),"SEG","TER","QUA","QUI","SEX","SAB","DOM")</f>
+        <v>DOM</v>
       </c>
       <c r="B14" s="112">
-        <v>3.4722222222222224E-2</v>
+        <v>0.58333333333333304</v>
       </c>
       <c r="C14" s="112">
-        <v>7.6388888888888895E-2</v>
+        <v>0.90625</v>
       </c>
       <c r="D14" s="110" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="E14" s="110" t="s">
         <v>103</v>
       </c>
       <c r="F14" s="110" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>SEX</v>
+        <v>DOM</v>
       </c>
       <c r="B15" s="112">
-        <v>3.4722222222222224E-2</v>
+        <v>0.58333333333333304</v>
       </c>
       <c r="C15" s="112">
-        <v>7.6388888888888895E-2</v>
+        <v>0.90625</v>
       </c>
       <c r="D15" s="110" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="E15" s="110" t="s">
         <v>104</v>
       </c>
       <c r="F15" s="110" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>SEX</v>
+        <v>DOM</v>
       </c>
       <c r="B16" s="112">
-        <v>3.4722222222222224E-2</v>
+        <v>0.58333333333333304</v>
       </c>
       <c r="C16" s="112">
-        <v>7.6388888888888895E-2</v>
+        <v>0.90625</v>
       </c>
       <c r="D16" s="110" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="E16" s="110" t="s">
         <v>103</v>
       </c>
       <c r="F16" s="110" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="str">
         <f ca="1">CHOOSE(WEEKDAY(TODAY(),2),"SEG","TER","QUA","QUI","SEX","SAB","DOM")</f>
-        <v>SEX</v>
+        <v>DOM</v>
       </c>
       <c r="B17" s="112">
-        <v>3.4722222222222224E-2</v>
+        <v>0.58333333333333304</v>
       </c>
       <c r="C17" s="112">
-        <v>7.6388888888888895E-2</v>
+        <v>0.90625</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="E17" s="1" t="s">
         <v>95</v>
@@ -5507,79 +5488,79 @@
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="str">
         <f ca="1">CHOOSE(WEEKDAY(TODAY(),2),"SEG","TER","QUA","QUI","SEX","SAB","DOM")</f>
-        <v>SEX</v>
+        <v>DOM</v>
       </c>
       <c r="B18" s="112">
-        <v>3.4722222222222224E-2</v>
+        <v>0.625</v>
       </c>
       <c r="C18" s="112">
-        <v>7.6388888888888895E-2</v>
+        <v>0.90625</v>
       </c>
       <c r="D18" s="110" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="E18" s="110" t="s">
         <v>102</v>
       </c>
       <c r="F18" s="110" t="s">
-        <v>108</v>
+        <v>96</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>SEX</v>
+        <v>DOM</v>
       </c>
       <c r="B19" s="112">
-        <v>7.6388888888888895E-2</v>
+        <v>0.625</v>
       </c>
       <c r="C19" s="112">
-        <v>0.118055555555556</v>
+        <v>0.90625</v>
       </c>
       <c r="D19" s="110" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="E19" s="110" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F19" s="110" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>SEX</v>
+        <v>DOM</v>
       </c>
       <c r="B20" s="112">
-        <v>7.6388888888888895E-2</v>
+        <v>0.625</v>
       </c>
       <c r="C20" s="112">
-        <v>0.118055555555556</v>
+        <v>0.90625</v>
       </c>
       <c r="D20" s="110" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="E20" s="110" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F20" s="110" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>SEX</v>
+        <v>DOM</v>
       </c>
       <c r="B21" s="112">
-        <v>7.6388888888888895E-2</v>
+        <v>0.625</v>
       </c>
       <c r="C21" s="112">
-        <v>0.118055555555556</v>
+        <v>0.90625</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>95</v>
@@ -5591,16 +5572,16 @@
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>SEX</v>
+        <v>DOM</v>
       </c>
       <c r="B22" s="112">
-        <v>7.6388888888888895E-2</v>
+        <v>0.625</v>
       </c>
       <c r="C22" s="112">
-        <v>0.118055555555556</v>
+        <v>0.90625</v>
       </c>
       <c r="D22" s="110" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="E22" s="110" t="s">
         <v>102</v>
@@ -5612,78 +5593,107 @@
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>SEX</v>
+        <v>DOM</v>
       </c>
       <c r="B23" s="112">
-        <v>7.6388888888888895E-2</v>
+        <v>0.66666666666666696</v>
       </c>
       <c r="C23" s="112">
-        <v>0.118055555555556</v>
+        <v>0.90625</v>
       </c>
       <c r="D23" s="110" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="E23" s="110" t="s">
         <v>103</v>
       </c>
       <c r="F23" s="110" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>SEX</v>
+        <v>DOM</v>
       </c>
       <c r="B24" s="112">
-        <v>7.6388888888888895E-2</v>
+        <v>0.66666666666666696</v>
       </c>
       <c r="C24" s="112">
-        <v>0.118055555555556</v>
+        <v>0.90625</v>
       </c>
       <c r="D24" s="110" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="E24" s="110" t="s">
         <v>104</v>
       </c>
       <c r="F24" s="110" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>SEX</v>
+        <v>DOM</v>
       </c>
       <c r="B25" s="112">
-        <v>7.6388888888888895E-2</v>
+        <v>0.66666666666666696</v>
       </c>
       <c r="C25" s="112">
-        <v>0.118055555555556</v>
+        <v>0.90625</v>
       </c>
       <c r="D25" s="110" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="E25" s="110" t="s">
         <v>103</v>
       </c>
       <c r="F25" s="110" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A26" s="1"/>
-      <c r="B26" s="112"/>
-      <c r="C26" s="112"/>
-      <c r="D26" s="1"/>
-      <c r="E26" s="1"/>
-      <c r="F26" s="1"/>
+      <c r="A26" s="1" t="str">
+        <f t="shared" ca="1" si="1"/>
+        <v>DOM</v>
+      </c>
+      <c r="B26" s="112">
+        <v>0.66666666666666696</v>
+      </c>
+      <c r="C26" s="112">
+        <v>0.90625</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>96</v>
+      </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A27" s="1"/>
-      <c r="B27" s="112"/>
-      <c r="C27" s="112"/>
+      <c r="A27" s="1" t="str">
+        <f t="shared" ca="1" si="1"/>
+        <v>DOM</v>
+      </c>
+      <c r="B27" s="112">
+        <v>0.66666666666666696</v>
+      </c>
+      <c r="C27" s="112">
+        <v>0.90625</v>
+      </c>
+      <c r="D27" s="110" t="s">
+        <v>107</v>
+      </c>
+      <c r="E27" s="110" t="s">
+        <v>102</v>
+      </c>
+      <c r="F27" s="110" t="s">
+        <v>96</v>
+      </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="1"/>
@@ -5950,1574 +5960,4 @@
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9DB064EE-8644-4CD1-8B51-D291BD535C03}">
-  <dimension ref="A1:F74"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="3" width="10.7109375" style="110" customWidth="1"/>
-    <col min="4" max="5" width="18.7109375" style="110" customWidth="1"/>
-    <col min="6" max="6" width="10.7109375" style="110" customWidth="1"/>
-    <col min="7" max="16384" width="9.140625" style="110"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="111" t="s">
-        <v>97</v>
-      </c>
-      <c r="B1" s="111" t="s">
-        <v>98</v>
-      </c>
-      <c r="C1" s="111" t="s">
-        <v>99</v>
-      </c>
-      <c r="D1" s="111" t="s">
-        <v>23</v>
-      </c>
-      <c r="E1" s="111" t="s">
-        <v>100</v>
-      </c>
-      <c r="F1" s="111" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="str">
-        <f ca="1">CHOOSE(WEEKDAY(TODAY(),2),"SEG","TER","QUA","QUI","SEX","SAB","DOM")</f>
-        <v>SEX</v>
-      </c>
-      <c r="B2" s="112">
-        <v>4.1666666666666664E-2</v>
-      </c>
-      <c r="C2" s="112">
-        <v>8.3333333333333329E-2</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="str">
-        <f ca="1">CHOOSE(WEEKDAY(TODAY(),2),"SEG","TER","QUA","QUI","SEX","SAB","DOM")</f>
-        <v>SEX</v>
-      </c>
-      <c r="B3" s="112">
-        <v>4.1666666666666664E-2</v>
-      </c>
-      <c r="C3" s="112">
-        <v>6.25E-2</v>
-      </c>
-      <c r="D3" s="110" t="s">
-        <v>110</v>
-      </c>
-      <c r="E3" s="110" t="s">
-        <v>102</v>
-      </c>
-      <c r="F3" s="110" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="str">
-        <f t="shared" ref="A4:A30" ca="1" si="0">CHOOSE(WEEKDAY(TODAY(),2),"SEG","TER","QUA","QUI","SEX","SAB","DOM")</f>
-        <v>SEX</v>
-      </c>
-      <c r="B4" s="112">
-        <v>4.1666666666666664E-2</v>
-      </c>
-      <c r="C4" s="112">
-        <v>6.25E-2</v>
-      </c>
-      <c r="D4" s="110" t="s">
-        <v>111</v>
-      </c>
-      <c r="E4" s="110" t="s">
-        <v>103</v>
-      </c>
-      <c r="F4" s="110" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="str">
-        <f t="shared" ca="1" si="0"/>
-        <v>SEX</v>
-      </c>
-      <c r="B5" s="112">
-        <v>4.1666666666666664E-2</v>
-      </c>
-      <c r="C5" s="112">
-        <v>6.25E-2</v>
-      </c>
-      <c r="D5" s="110" t="s">
-        <v>112</v>
-      </c>
-      <c r="E5" s="110" t="s">
-        <v>104</v>
-      </c>
-      <c r="F5" s="110" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="str">
-        <f t="shared" ca="1" si="0"/>
-        <v>SEX</v>
-      </c>
-      <c r="B6" s="112">
-        <v>4.1666666666666664E-2</v>
-      </c>
-      <c r="C6" s="112">
-        <v>6.25E-2</v>
-      </c>
-      <c r="D6" s="110" t="s">
-        <v>113</v>
-      </c>
-      <c r="E6" s="110" t="s">
-        <v>105</v>
-      </c>
-      <c r="F6" s="110" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="str">
-        <f t="shared" ca="1" si="0"/>
-        <v>SEX</v>
-      </c>
-      <c r="B7" s="112">
-        <v>4.1666666666666664E-2</v>
-      </c>
-      <c r="C7" s="112">
-        <v>6.25E-2</v>
-      </c>
-      <c r="D7" s="110" t="s">
-        <v>114</v>
-      </c>
-      <c r="E7" s="110" t="s">
-        <v>106</v>
-      </c>
-      <c r="F7" s="110" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="str">
-        <f t="shared" ca="1" si="0"/>
-        <v>SEX</v>
-      </c>
-      <c r="B8" s="112">
-        <v>4.1666666666666664E-2</v>
-      </c>
-      <c r="C8" s="112">
-        <v>6.25E-2</v>
-      </c>
-      <c r="D8" s="110" t="s">
-        <v>115</v>
-      </c>
-      <c r="E8" s="110" t="s">
-        <v>107</v>
-      </c>
-      <c r="F8" s="110" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="str">
-        <f t="shared" ca="1" si="0"/>
-        <v>SEX</v>
-      </c>
-      <c r="B9" s="112">
-        <v>6.25E-2</v>
-      </c>
-      <c r="C9" s="112">
-        <v>0.104166666666667</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="F9" s="1" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="str">
-        <f t="shared" ca="1" si="0"/>
-        <v>SEX</v>
-      </c>
-      <c r="B10" s="112">
-        <v>6.25E-2</v>
-      </c>
-      <c r="C10" s="112">
-        <v>0.104166666666667</v>
-      </c>
-      <c r="D10" s="110" t="s">
-        <v>110</v>
-      </c>
-      <c r="E10" s="110" t="s">
-        <v>102</v>
-      </c>
-      <c r="F10" s="110" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="str">
-        <f t="shared" ca="1" si="0"/>
-        <v>SEX</v>
-      </c>
-      <c r="B11" s="112">
-        <v>6.25E-2</v>
-      </c>
-      <c r="C11" s="112">
-        <v>0.104166666666667</v>
-      </c>
-      <c r="D11" s="110" t="s">
-        <v>111</v>
-      </c>
-      <c r="E11" s="110" t="s">
-        <v>103</v>
-      </c>
-      <c r="F11" s="110" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="str">
-        <f t="shared" ca="1" si="0"/>
-        <v>SEX</v>
-      </c>
-      <c r="B12" s="112">
-        <v>6.25E-2</v>
-      </c>
-      <c r="C12" s="112">
-        <v>0.104166666666667</v>
-      </c>
-      <c r="D12" s="110" t="s">
-        <v>112</v>
-      </c>
-      <c r="E12" s="110" t="s">
-        <v>104</v>
-      </c>
-      <c r="F12" s="110" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="str">
-        <f t="shared" ca="1" si="0"/>
-        <v>SEX</v>
-      </c>
-      <c r="B13" s="112">
-        <v>6.25E-2</v>
-      </c>
-      <c r="C13" s="112">
-        <v>0.104166666666667</v>
-      </c>
-      <c r="D13" s="110" t="s">
-        <v>113</v>
-      </c>
-      <c r="E13" s="110" t="s">
-        <v>105</v>
-      </c>
-      <c r="F13" s="110" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="str">
-        <f t="shared" ca="1" si="0"/>
-        <v>SEX</v>
-      </c>
-      <c r="B14" s="112">
-        <v>6.25E-2</v>
-      </c>
-      <c r="C14" s="112">
-        <v>0.104166666666667</v>
-      </c>
-      <c r="D14" s="110" t="s">
-        <v>114</v>
-      </c>
-      <c r="E14" s="110" t="s">
-        <v>106</v>
-      </c>
-      <c r="F14" s="110" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="str">
-        <f t="shared" ca="1" si="0"/>
-        <v>SEX</v>
-      </c>
-      <c r="B15" s="112">
-        <v>6.25E-2</v>
-      </c>
-      <c r="C15" s="112">
-        <v>0.104166666666667</v>
-      </c>
-      <c r="D15" s="110" t="s">
-        <v>115</v>
-      </c>
-      <c r="E15" s="110" t="s">
-        <v>107</v>
-      </c>
-      <c r="F15" s="110" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="str">
-        <f t="shared" ca="1" si="0"/>
-        <v>SEX</v>
-      </c>
-      <c r="B16" s="112">
-        <v>4.1666666666666664E-2</v>
-      </c>
-      <c r="C16" s="112">
-        <v>8.3333333333333329E-2</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="F16" s="1" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="str">
-        <f t="shared" ca="1" si="0"/>
-        <v>SEX</v>
-      </c>
-      <c r="B17" s="112">
-        <v>4.1666666666666664E-2</v>
-      </c>
-      <c r="C17" s="112">
-        <v>6.25E-2</v>
-      </c>
-      <c r="D17" s="110" t="s">
-        <v>110</v>
-      </c>
-      <c r="E17" s="110" t="s">
-        <v>102</v>
-      </c>
-      <c r="F17" s="110" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="str">
-        <f t="shared" ca="1" si="0"/>
-        <v>SEX</v>
-      </c>
-      <c r="B18" s="112">
-        <v>4.1666666666666664E-2</v>
-      </c>
-      <c r="C18" s="112">
-        <v>6.25E-2</v>
-      </c>
-      <c r="D18" s="110" t="s">
-        <v>111</v>
-      </c>
-      <c r="E18" s="110" t="s">
-        <v>103</v>
-      </c>
-      <c r="F18" s="110" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="str">
-        <f t="shared" ca="1" si="0"/>
-        <v>SEX</v>
-      </c>
-      <c r="B19" s="112">
-        <v>4.1666666666666664E-2</v>
-      </c>
-      <c r="C19" s="112">
-        <v>6.25E-2</v>
-      </c>
-      <c r="D19" s="110" t="s">
-        <v>112</v>
-      </c>
-      <c r="E19" s="110" t="s">
-        <v>104</v>
-      </c>
-      <c r="F19" s="110" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="str">
-        <f t="shared" ca="1" si="0"/>
-        <v>SEX</v>
-      </c>
-      <c r="B20" s="112">
-        <v>4.1666666666666664E-2</v>
-      </c>
-      <c r="C20" s="112">
-        <v>6.25E-2</v>
-      </c>
-      <c r="D20" s="110" t="s">
-        <v>113</v>
-      </c>
-      <c r="E20" s="110" t="s">
-        <v>105</v>
-      </c>
-      <c r="F20" s="110" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="str">
-        <f t="shared" ca="1" si="0"/>
-        <v>SEX</v>
-      </c>
-      <c r="B21" s="112">
-        <v>4.1666666666666664E-2</v>
-      </c>
-      <c r="C21" s="112">
-        <v>6.25E-2</v>
-      </c>
-      <c r="D21" s="110" t="s">
-        <v>114</v>
-      </c>
-      <c r="E21" s="110" t="s">
-        <v>106</v>
-      </c>
-      <c r="F21" s="110" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22" s="1" t="str">
-        <f t="shared" ca="1" si="0"/>
-        <v>SEX</v>
-      </c>
-      <c r="B22" s="112">
-        <v>4.1666666666666664E-2</v>
-      </c>
-      <c r="C22" s="112">
-        <v>6.25E-2</v>
-      </c>
-      <c r="D22" s="110" t="s">
-        <v>115</v>
-      </c>
-      <c r="E22" s="110" t="s">
-        <v>107</v>
-      </c>
-      <c r="F22" s="110" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A23" s="1" t="str">
-        <f t="shared" ca="1" si="0"/>
-        <v>SEX</v>
-      </c>
-      <c r="B23" s="112">
-        <v>6.25E-2</v>
-      </c>
-      <c r="C23" s="112">
-        <v>0.104166666666667</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="E23" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="F23" s="1" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A24" s="1" t="str">
-        <f t="shared" ca="1" si="0"/>
-        <v>SEX</v>
-      </c>
-      <c r="B24" s="112">
-        <v>6.25E-2</v>
-      </c>
-      <c r="C24" s="112">
-        <v>0.104166666666667</v>
-      </c>
-      <c r="D24" s="110" t="s">
-        <v>110</v>
-      </c>
-      <c r="E24" s="110" t="s">
-        <v>102</v>
-      </c>
-      <c r="F24" s="110" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A25" s="1" t="str">
-        <f t="shared" ca="1" si="0"/>
-        <v>SEX</v>
-      </c>
-      <c r="B25" s="112">
-        <v>6.25E-2</v>
-      </c>
-      <c r="C25" s="112">
-        <v>0.104166666666667</v>
-      </c>
-      <c r="D25" s="110" t="s">
-        <v>111</v>
-      </c>
-      <c r="E25" s="110" t="s">
-        <v>103</v>
-      </c>
-      <c r="F25" s="110" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A26" s="1" t="str">
-        <f t="shared" ca="1" si="0"/>
-        <v>SEX</v>
-      </c>
-      <c r="B26" s="112">
-        <v>6.25E-2</v>
-      </c>
-      <c r="C26" s="112">
-        <v>0.104166666666667</v>
-      </c>
-      <c r="D26" s="110" t="s">
-        <v>112</v>
-      </c>
-      <c r="E26" s="110" t="s">
-        <v>104</v>
-      </c>
-      <c r="F26" s="110" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A27" s="1" t="str">
-        <f t="shared" ca="1" si="0"/>
-        <v>SEX</v>
-      </c>
-      <c r="B27" s="112">
-        <v>6.25E-2</v>
-      </c>
-      <c r="C27" s="112">
-        <v>0.104166666666667</v>
-      </c>
-      <c r="D27" s="110" t="s">
-        <v>113</v>
-      </c>
-      <c r="E27" s="110" t="s">
-        <v>105</v>
-      </c>
-      <c r="F27" s="110" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" s="1" t="str">
-        <f t="shared" ca="1" si="0"/>
-        <v>SEX</v>
-      </c>
-      <c r="B28" s="112">
-        <v>6.25E-2</v>
-      </c>
-      <c r="C28" s="112">
-        <v>0.104166666666667</v>
-      </c>
-      <c r="D28" s="110" t="s">
-        <v>114</v>
-      </c>
-      <c r="E28" s="110" t="s">
-        <v>106</v>
-      </c>
-      <c r="F28" s="110" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A29" s="1" t="str">
-        <f t="shared" ca="1" si="0"/>
-        <v>SEX</v>
-      </c>
-      <c r="B29" s="112">
-        <v>6.25E-2</v>
-      </c>
-      <c r="C29" s="112">
-        <v>0.104166666666667</v>
-      </c>
-      <c r="D29" s="110" t="s">
-        <v>115</v>
-      </c>
-      <c r="E29" s="110" t="s">
-        <v>107</v>
-      </c>
-      <c r="F29" s="110" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A30" s="1" t="str">
-        <f t="shared" ca="1" si="0"/>
-        <v>SEX</v>
-      </c>
-      <c r="B30" s="112">
-        <v>4.1666666666666664E-2</v>
-      </c>
-      <c r="C30" s="112">
-        <v>8.3333333333333329E-2</v>
-      </c>
-      <c r="D30" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="E30" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="F30" s="1" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A31" s="1" t="str">
-        <f ca="1">CHOOSE(WEEKDAY(TODAY(),2),"SEG","TER","QUA","QUI","SEX","SAB","DOM")</f>
-        <v>SEX</v>
-      </c>
-      <c r="B31" s="112">
-        <v>4.1666666666666664E-2</v>
-      </c>
-      <c r="C31" s="112">
-        <v>8.3333333333333329E-2</v>
-      </c>
-      <c r="D31" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="E31" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="F31" s="1" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A32" s="1" t="str">
-        <f ca="1">CHOOSE(WEEKDAY(TODAY(),2),"SEG","TER","QUA","QUI","SEX","SAB","DOM")</f>
-        <v>SEX</v>
-      </c>
-      <c r="B32" s="112">
-        <v>4.1666666666666664E-2</v>
-      </c>
-      <c r="C32" s="112">
-        <v>6.25E-2</v>
-      </c>
-      <c r="D32" s="110" t="s">
-        <v>110</v>
-      </c>
-      <c r="E32" s="110" t="s">
-        <v>102</v>
-      </c>
-      <c r="F32" s="110" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A33" s="1" t="str">
-        <f t="shared" ref="A33:A74" ca="1" si="1">CHOOSE(WEEKDAY(TODAY(),2),"SEG","TER","QUA","QUI","SEX","SAB","DOM")</f>
-        <v>SEX</v>
-      </c>
-      <c r="B33" s="112">
-        <v>4.1666666666666664E-2</v>
-      </c>
-      <c r="C33" s="112">
-        <v>6.25E-2</v>
-      </c>
-      <c r="D33" s="110" t="s">
-        <v>111</v>
-      </c>
-      <c r="E33" s="110" t="s">
-        <v>103</v>
-      </c>
-      <c r="F33" s="110" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A34" s="1" t="str">
-        <f t="shared" ca="1" si="1"/>
-        <v>SEX</v>
-      </c>
-      <c r="B34" s="112">
-        <v>4.1666666666666664E-2</v>
-      </c>
-      <c r="C34" s="112">
-        <v>6.25E-2</v>
-      </c>
-      <c r="D34" s="110" t="s">
-        <v>112</v>
-      </c>
-      <c r="E34" s="110" t="s">
-        <v>104</v>
-      </c>
-      <c r="F34" s="110" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A35" s="1" t="str">
-        <f t="shared" ca="1" si="1"/>
-        <v>SEX</v>
-      </c>
-      <c r="B35" s="112">
-        <v>4.1666666666666664E-2</v>
-      </c>
-      <c r="C35" s="112">
-        <v>6.25E-2</v>
-      </c>
-      <c r="D35" s="110" t="s">
-        <v>113</v>
-      </c>
-      <c r="E35" s="110" t="s">
-        <v>105</v>
-      </c>
-      <c r="F35" s="110" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A36" s="1" t="str">
-        <f t="shared" ca="1" si="1"/>
-        <v>SEX</v>
-      </c>
-      <c r="B36" s="112">
-        <v>4.1666666666666664E-2</v>
-      </c>
-      <c r="C36" s="112">
-        <v>6.25E-2</v>
-      </c>
-      <c r="D36" s="110" t="s">
-        <v>115</v>
-      </c>
-      <c r="E36" s="110" t="s">
-        <v>106</v>
-      </c>
-      <c r="F36" s="110" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A37" s="1" t="str">
-        <f t="shared" ca="1" si="1"/>
-        <v>SEX</v>
-      </c>
-      <c r="B37" s="112">
-        <v>4.1666666666666664E-2</v>
-      </c>
-      <c r="C37" s="112">
-        <v>6.25E-2</v>
-      </c>
-      <c r="D37" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="E37" s="110" t="s">
-        <v>107</v>
-      </c>
-      <c r="F37" s="110" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A38" s="1" t="str">
-        <f t="shared" ca="1" si="1"/>
-        <v>SEX</v>
-      </c>
-      <c r="B38" s="112">
-        <v>6.25E-2</v>
-      </c>
-      <c r="C38" s="112">
-        <v>0.104166666666667</v>
-      </c>
-      <c r="D38" s="110" t="s">
-        <v>110</v>
-      </c>
-      <c r="E38" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="F38" s="1" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A39" s="1" t="str">
-        <f t="shared" ca="1" si="1"/>
-        <v>SEX</v>
-      </c>
-      <c r="B39" s="112">
-        <v>6.25E-2</v>
-      </c>
-      <c r="C39" s="112">
-        <v>0.104166666666667</v>
-      </c>
-      <c r="D39" s="110" t="s">
-        <v>111</v>
-      </c>
-      <c r="E39" s="110" t="s">
-        <v>102</v>
-      </c>
-      <c r="F39" s="110" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A40" s="1" t="str">
-        <f t="shared" ca="1" si="1"/>
-        <v>SEX</v>
-      </c>
-      <c r="B40" s="112">
-        <v>6.25E-2</v>
-      </c>
-      <c r="C40" s="112">
-        <v>0.104166666666667</v>
-      </c>
-      <c r="D40" s="110" t="s">
-        <v>112</v>
-      </c>
-      <c r="E40" s="110" t="s">
-        <v>103</v>
-      </c>
-      <c r="F40" s="110" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A41" s="1" t="str">
-        <f t="shared" ca="1" si="1"/>
-        <v>SEX</v>
-      </c>
-      <c r="B41" s="112">
-        <v>0.104166666666667</v>
-      </c>
-      <c r="C41" s="112">
-        <v>0.14583333333333401</v>
-      </c>
-      <c r="D41" s="110" t="s">
-        <v>113</v>
-      </c>
-      <c r="E41" s="110" t="s">
-        <v>102</v>
-      </c>
-      <c r="F41" s="110" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A42" s="1" t="str">
-        <f t="shared" ca="1" si="1"/>
-        <v>SEX</v>
-      </c>
-      <c r="B42" s="112">
-        <v>0.104166666666667</v>
-      </c>
-      <c r="C42" s="112">
-        <v>0.14583333333333401</v>
-      </c>
-      <c r="D42" s="110" t="s">
-        <v>114</v>
-      </c>
-      <c r="E42" s="110" t="s">
-        <v>103</v>
-      </c>
-      <c r="F42" s="110" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A43" s="1" t="str">
-        <f t="shared" ca="1" si="1"/>
-        <v>SEX</v>
-      </c>
-      <c r="B43" s="112">
-        <v>0.104166666666667</v>
-      </c>
-      <c r="C43" s="112">
-        <v>0.14583333333333401</v>
-      </c>
-      <c r="D43" s="110" t="s">
-        <v>115</v>
-      </c>
-      <c r="E43" s="110" t="s">
-        <v>104</v>
-      </c>
-      <c r="F43" s="110" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A44" s="1" t="str">
-        <f t="shared" ca="1" si="1"/>
-        <v>SEX</v>
-      </c>
-      <c r="B44" s="112">
-        <v>0.104166666666667</v>
-      </c>
-      <c r="C44" s="112">
-        <v>0.14583333333333401</v>
-      </c>
-      <c r="D44" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="E44" s="110" t="s">
-        <v>105</v>
-      </c>
-      <c r="F44" s="110" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A45" s="1" t="str">
-        <f t="shared" ca="1" si="1"/>
-        <v>SEX</v>
-      </c>
-      <c r="B45" s="112">
-        <v>0.104166666666667</v>
-      </c>
-      <c r="C45" s="112">
-        <v>0.14583333333333401</v>
-      </c>
-      <c r="D45" s="110" t="s">
-        <v>110</v>
-      </c>
-      <c r="E45" s="110" t="s">
-        <v>106</v>
-      </c>
-      <c r="F45" s="110" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A46" s="1" t="str">
-        <f t="shared" ca="1" si="1"/>
-        <v>SEX</v>
-      </c>
-      <c r="B46" s="112">
-        <v>0.104166666666667</v>
-      </c>
-      <c r="C46" s="112">
-        <v>0.14583333333333401</v>
-      </c>
-      <c r="D46" s="110" t="s">
-        <v>111</v>
-      </c>
-      <c r="E46" s="110" t="s">
-        <v>107</v>
-      </c>
-      <c r="F46" s="110" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A47" s="1" t="str">
-        <f t="shared" ca="1" si="1"/>
-        <v>SEX</v>
-      </c>
-      <c r="B47" s="112">
-        <v>0.104166666666667</v>
-      </c>
-      <c r="C47" s="112">
-        <v>0.14583333333333401</v>
-      </c>
-      <c r="D47" s="110" t="s">
-        <v>112</v>
-      </c>
-      <c r="E47" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="F47" s="1" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A48" s="1" t="str">
-        <f t="shared" ca="1" si="1"/>
-        <v>SEX</v>
-      </c>
-      <c r="B48" s="112">
-        <v>0.104166666666667</v>
-      </c>
-      <c r="C48" s="112">
-        <v>0.14583333333333401</v>
-      </c>
-      <c r="D48" s="110" t="s">
-        <v>113</v>
-      </c>
-      <c r="E48" s="110" t="s">
-        <v>102</v>
-      </c>
-      <c r="F48" s="110" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A49" s="1" t="str">
-        <f t="shared" ca="1" si="1"/>
-        <v>SEX</v>
-      </c>
-      <c r="B49" s="112">
-        <v>0.104166666666667</v>
-      </c>
-      <c r="C49" s="112">
-        <v>0.14583333333333401</v>
-      </c>
-      <c r="D49" s="110" t="s">
-        <v>114</v>
-      </c>
-      <c r="E49" s="110" t="s">
-        <v>103</v>
-      </c>
-      <c r="F49" s="110" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A50" s="1" t="str">
-        <f t="shared" ca="1" si="1"/>
-        <v>SEX</v>
-      </c>
-      <c r="B50" s="112">
-        <v>0.104166666666667</v>
-      </c>
-      <c r="C50" s="112">
-        <v>0.14583333333333401</v>
-      </c>
-      <c r="D50" s="110" t="s">
-        <v>115</v>
-      </c>
-      <c r="E50" s="110" t="s">
-        <v>104</v>
-      </c>
-      <c r="F50" s="110" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A51" s="1" t="str">
-        <f t="shared" ca="1" si="1"/>
-        <v>SEX</v>
-      </c>
-      <c r="B51" s="112">
-        <v>0.104166666666667</v>
-      </c>
-      <c r="C51" s="112">
-        <v>0.14583333333333401</v>
-      </c>
-      <c r="D51" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="E51" s="110" t="s">
-        <v>105</v>
-      </c>
-      <c r="F51" s="110" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A52" s="1" t="str">
-        <f t="shared" ca="1" si="1"/>
-        <v>SEX</v>
-      </c>
-      <c r="B52" s="112">
-        <v>0.104166666666667</v>
-      </c>
-      <c r="C52" s="112">
-        <v>0.14583333333333401</v>
-      </c>
-      <c r="D52" s="110" t="s">
-        <v>110</v>
-      </c>
-      <c r="E52" s="110" t="s">
-        <v>106</v>
-      </c>
-      <c r="F52" s="110" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A53" s="1" t="str">
-        <f t="shared" ca="1" si="1"/>
-        <v>SEX</v>
-      </c>
-      <c r="B53" s="112">
-        <v>0.104166666666667</v>
-      </c>
-      <c r="C53" s="112">
-        <v>0.14583333333333401</v>
-      </c>
-      <c r="D53" s="110" t="s">
-        <v>111</v>
-      </c>
-      <c r="E53" s="110" t="s">
-        <v>107</v>
-      </c>
-      <c r="F53" s="110" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A54" s="1" t="str">
-        <f t="shared" ca="1" si="1"/>
-        <v>SEX</v>
-      </c>
-      <c r="B54" s="112">
-        <v>0.104166666666667</v>
-      </c>
-      <c r="C54" s="112">
-        <v>0.14583333333333401</v>
-      </c>
-      <c r="D54" s="110" t="s">
-        <v>112</v>
-      </c>
-      <c r="E54" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="F54" s="1" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A55" s="1" t="str">
-        <f t="shared" ca="1" si="1"/>
-        <v>SEX</v>
-      </c>
-      <c r="B55" s="112">
-        <v>0.104166666666667</v>
-      </c>
-      <c r="C55" s="112">
-        <v>0.14583333333333401</v>
-      </c>
-      <c r="D55" s="110" t="s">
-        <v>113</v>
-      </c>
-      <c r="E55" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="F55" s="1" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A56" s="1" t="str">
-        <f t="shared" ca="1" si="1"/>
-        <v>SEX</v>
-      </c>
-      <c r="B56" s="112">
-        <v>0.104166666666667</v>
-      </c>
-      <c r="C56" s="112">
-        <v>0.14583333333333401</v>
-      </c>
-      <c r="D56" s="110" t="s">
-        <v>114</v>
-      </c>
-      <c r="E56" s="110" t="s">
-        <v>102</v>
-      </c>
-      <c r="F56" s="110" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A57" s="1" t="str">
-        <f t="shared" ca="1" si="1"/>
-        <v>SEX</v>
-      </c>
-      <c r="B57" s="112">
-        <v>0.104166666666667</v>
-      </c>
-      <c r="C57" s="112">
-        <v>0.14583333333333401</v>
-      </c>
-      <c r="D57" s="110" t="s">
-        <v>115</v>
-      </c>
-      <c r="E57" s="110" t="s">
-        <v>103</v>
-      </c>
-      <c r="F57" s="110" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A58" s="1" t="str">
-        <f t="shared" ca="1" si="1"/>
-        <v>SEX</v>
-      </c>
-      <c r="B58" s="112">
-        <v>0.104166666666667</v>
-      </c>
-      <c r="C58" s="112">
-        <v>0.14583333333333401</v>
-      </c>
-      <c r="D58" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="E58" s="110" t="s">
-        <v>104</v>
-      </c>
-      <c r="F58" s="110" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A59" s="1" t="str">
-        <f t="shared" ca="1" si="1"/>
-        <v>SEX</v>
-      </c>
-      <c r="B59" s="112">
-        <v>0.104166666666667</v>
-      </c>
-      <c r="C59" s="112">
-        <v>0.14583333333333401</v>
-      </c>
-      <c r="D59" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="E59" s="110" t="s">
-        <v>105</v>
-      </c>
-      <c r="F59" s="110" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A60" s="1" t="str">
-        <f t="shared" ca="1" si="1"/>
-        <v>SEX</v>
-      </c>
-      <c r="B60" s="112">
-        <v>0.104166666666667</v>
-      </c>
-      <c r="C60" s="112">
-        <v>0.14583333333333401</v>
-      </c>
-      <c r="D60" s="110" t="s">
-        <v>110</v>
-      </c>
-      <c r="E60" s="110" t="s">
-        <v>106</v>
-      </c>
-      <c r="F60" s="110" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A61" s="1" t="str">
-        <f t="shared" ca="1" si="1"/>
-        <v>SEX</v>
-      </c>
-      <c r="B61" s="112">
-        <v>0.104166666666667</v>
-      </c>
-      <c r="C61" s="112">
-        <v>0.14583333333333401</v>
-      </c>
-      <c r="D61" s="110" t="s">
-        <v>111</v>
-      </c>
-      <c r="E61" s="110" t="s">
-        <v>107</v>
-      </c>
-      <c r="F61" s="110" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A62" s="1" t="str">
-        <f t="shared" ca="1" si="1"/>
-        <v>SEX</v>
-      </c>
-      <c r="B62" s="112">
-        <v>0.104166666666667</v>
-      </c>
-      <c r="C62" s="112">
-        <v>0.14583333333333401</v>
-      </c>
-      <c r="D62" s="110" t="s">
-        <v>112</v>
-      </c>
-      <c r="E62" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="F62" s="1" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A63" s="1" t="str">
-        <f t="shared" ca="1" si="1"/>
-        <v>SEX</v>
-      </c>
-      <c r="B63" s="112">
-        <v>0.104166666666667</v>
-      </c>
-      <c r="C63" s="112">
-        <v>0.14583333333333401</v>
-      </c>
-      <c r="D63" s="110" t="s">
-        <v>113</v>
-      </c>
-      <c r="E63" s="110" t="s">
-        <v>102</v>
-      </c>
-      <c r="F63" s="110" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A64" s="1" t="str">
-        <f t="shared" ca="1" si="1"/>
-        <v>SEX</v>
-      </c>
-      <c r="B64" s="112">
-        <v>0.104166666666667</v>
-      </c>
-      <c r="C64" s="112">
-        <v>0.14583333333333401</v>
-      </c>
-      <c r="D64" s="110" t="s">
-        <v>115</v>
-      </c>
-      <c r="E64" s="110" t="s">
-        <v>103</v>
-      </c>
-      <c r="F64" s="110" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A65" s="1" t="str">
-        <f t="shared" ca="1" si="1"/>
-        <v>SEX</v>
-      </c>
-      <c r="B65" s="112">
-        <v>0.104166666666667</v>
-      </c>
-      <c r="C65" s="112">
-        <v>0.14583333333333401</v>
-      </c>
-      <c r="D65" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="E65" s="110" t="s">
-        <v>102</v>
-      </c>
-      <c r="F65" s="110" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A66" s="1" t="str">
-        <f t="shared" ca="1" si="1"/>
-        <v>SEX</v>
-      </c>
-      <c r="B66" s="112">
-        <v>0.104166666666667</v>
-      </c>
-      <c r="C66" s="112">
-        <v>0.14583333333333401</v>
-      </c>
-      <c r="D66" s="110" t="s">
-        <v>110</v>
-      </c>
-      <c r="E66" s="110" t="s">
-        <v>103</v>
-      </c>
-      <c r="F66" s="110" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A67" s="1" t="str">
-        <f t="shared" ca="1" si="1"/>
-        <v>SEX</v>
-      </c>
-      <c r="B67" s="112">
-        <v>0.104166666666667</v>
-      </c>
-      <c r="C67" s="112">
-        <v>0.14583333333333401</v>
-      </c>
-      <c r="D67" s="110" t="s">
-        <v>111</v>
-      </c>
-      <c r="E67" s="110" t="s">
-        <v>104</v>
-      </c>
-      <c r="F67" s="110" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A68" s="1" t="str">
-        <f t="shared" ca="1" si="1"/>
-        <v>SEX</v>
-      </c>
-      <c r="B68" s="112">
-        <v>0.104166666666667</v>
-      </c>
-      <c r="C68" s="112">
-        <v>0.14583333333333401</v>
-      </c>
-      <c r="D68" s="110" t="s">
-        <v>112</v>
-      </c>
-      <c r="E68" s="110" t="s">
-        <v>105</v>
-      </c>
-      <c r="F68" s="110" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A69" s="1" t="str">
-        <f t="shared" ca="1" si="1"/>
-        <v>SEX</v>
-      </c>
-      <c r="B69" s="112">
-        <v>0.104166666666667</v>
-      </c>
-      <c r="C69" s="112">
-        <v>0.14583333333333401</v>
-      </c>
-      <c r="D69" s="110" t="s">
-        <v>113</v>
-      </c>
-      <c r="E69" s="110" t="s">
-        <v>106</v>
-      </c>
-      <c r="F69" s="110" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A70" s="1" t="str">
-        <f t="shared" ca="1" si="1"/>
-        <v>SEX</v>
-      </c>
-      <c r="B70" s="112">
-        <v>0.104166666666667</v>
-      </c>
-      <c r="C70" s="112">
-        <v>0.14583333333333401</v>
-      </c>
-      <c r="D70" s="110" t="s">
-        <v>114</v>
-      </c>
-      <c r="E70" s="110" t="s">
-        <v>107</v>
-      </c>
-      <c r="F70" s="110" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A71" s="1" t="str">
-        <f t="shared" ca="1" si="1"/>
-        <v>SEX</v>
-      </c>
-      <c r="B71" s="112">
-        <v>0.104166666666667</v>
-      </c>
-      <c r="C71" s="112">
-        <v>0.14583333333333401</v>
-      </c>
-      <c r="D71" s="110" t="s">
-        <v>115</v>
-      </c>
-      <c r="E71" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="F71" s="1" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A72" s="1" t="str">
-        <f t="shared" ca="1" si="1"/>
-        <v>SEX</v>
-      </c>
-      <c r="B72" s="112">
-        <v>0.104166666666667</v>
-      </c>
-      <c r="C72" s="112">
-        <v>0.14583333333333401</v>
-      </c>
-      <c r="D72" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="E72" s="110" t="s">
-        <v>102</v>
-      </c>
-      <c r="F72" s="110" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A73" s="1" t="str">
-        <f t="shared" ca="1" si="1"/>
-        <v>SEX</v>
-      </c>
-      <c r="B73" s="112">
-        <v>0.104166666666667</v>
-      </c>
-      <c r="C73" s="112">
-        <v>0.14583333333333401</v>
-      </c>
-      <c r="D73" s="110" t="s">
-        <v>110</v>
-      </c>
-      <c r="E73" s="110" t="s">
-        <v>103</v>
-      </c>
-      <c r="F73" s="110" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A74" s="1" t="str">
-        <f t="shared" ca="1" si="1"/>
-        <v>SEX</v>
-      </c>
-      <c r="B74" s="112">
-        <v>0.104166666666667</v>
-      </c>
-      <c r="C74" s="112">
-        <v>0.14583333333333401</v>
-      </c>
-      <c r="D74" s="110" t="s">
-        <v>111</v>
-      </c>
-      <c r="E74" s="110" t="s">
-        <v>104</v>
-      </c>
-      <c r="F74" s="110" t="s">
-        <v>108</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Extract Excel reload flow into xlsx loader
Move Excel reload responsibility out of clubal.py into infra.xlsx_loader by introducing reload_classes_if_needed. Keep the main file as a thin orchestration layer while preserving the existing reload behavior, file mtime checks, and XLSX logging output.
</commit_message>
<xml_diff>
--- a/grade.xlsx
+++ b/grade.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrativo\Documents\GitHub\clubal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F8AC58B-4057-4A83-BC40-046A4FDE9636}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{532C5FBE-C8CC-4EDA-AC74-96C05184073D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1499,19 +1499,40 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="20" fontId="5" fillId="9" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="9" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="2" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="8" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="8" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="2" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="20" fontId="5" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1520,27 +1541,54 @@
     <xf numFmtId="20" fontId="5" fillId="2" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="20" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="20" fontId="5" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="20" fontId="5" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="9" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="20" fontId="5" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="20" fontId="5" fillId="9" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="9" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="9" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1550,67 +1598,19 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="2" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="9" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="9" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="8" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="8" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="9" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="9" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="2" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1640,81 +1640,6 @@
     <xf numFmtId="0" fontId="5" fillId="9" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="7" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
@@ -1740,6 +1665,81 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="7" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2834,7 +2834,7 @@
       <c r="B4" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="C4" s="117" t="s">
+      <c r="C4" s="150" t="s">
         <v>24</v>
       </c>
       <c r="D4" s="114"/>
@@ -2846,23 +2846,23 @@
         <v>4</v>
       </c>
       <c r="H4" s="114"/>
-      <c r="I4" s="120" t="s">
+      <c r="I4" s="153" t="s">
         <v>5</v>
       </c>
-      <c r="J4" s="121"/>
-      <c r="K4" s="118" t="s">
+      <c r="J4" s="154"/>
+      <c r="K4" s="151" t="s">
         <v>6</v>
       </c>
-      <c r="L4" s="119"/>
-      <c r="M4" s="118" t="s">
+      <c r="L4" s="152"/>
+      <c r="M4" s="151" t="s">
         <v>35</v>
       </c>
-      <c r="N4" s="119"/>
+      <c r="N4" s="152"/>
       <c r="O4" s="2"/>
     </row>
     <row r="5" spans="1:15" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2"/>
-      <c r="B5" s="136" t="s">
+      <c r="B5" s="137" t="s">
         <v>22</v>
       </c>
       <c r="C5" s="140" t="s">
@@ -2893,15 +2893,15 @@
       <c r="L5" s="41">
         <v>0.45833333333333331</v>
       </c>
-      <c r="M5" s="145"/>
-      <c r="N5" s="146"/>
+      <c r="M5" s="125"/>
+      <c r="N5" s="126"/>
       <c r="O5" s="2"/>
     </row>
     <row r="6" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A6" s="2"/>
-      <c r="B6" s="137"/>
-      <c r="C6" s="128"/>
-      <c r="D6" s="129"/>
+      <c r="B6" s="138"/>
+      <c r="C6" s="142"/>
+      <c r="D6" s="143"/>
       <c r="E6" s="45">
         <v>0.73958333333333337</v>
       </c>
@@ -2918,17 +2918,17 @@
       </c>
       <c r="K6" s="45"/>
       <c r="L6" s="46"/>
-      <c r="M6" s="147"/>
-      <c r="N6" s="148"/>
+      <c r="M6" s="117"/>
+      <c r="N6" s="118"/>
       <c r="O6" s="2"/>
     </row>
     <row r="7" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
-      <c r="B7" s="137"/>
-      <c r="C7" s="128" t="s">
+      <c r="B7" s="138"/>
+      <c r="C7" s="142" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="129"/>
+      <c r="D7" s="143"/>
       <c r="E7" s="40">
         <v>0.42708333333333331</v>
       </c>
@@ -2945,15 +2945,15 @@
       </c>
       <c r="K7" s="40"/>
       <c r="L7" s="41"/>
-      <c r="M7" s="145"/>
-      <c r="N7" s="146"/>
+      <c r="M7" s="125"/>
+      <c r="N7" s="126"/>
       <c r="O7" s="2"/>
     </row>
     <row r="8" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A8" s="2"/>
-      <c r="B8" s="137"/>
-      <c r="C8" s="128"/>
-      <c r="D8" s="129"/>
+      <c r="B8" s="138"/>
+      <c r="C8" s="142"/>
+      <c r="D8" s="143"/>
       <c r="E8" s="45">
         <v>0.77083333333333337</v>
       </c>
@@ -2970,17 +2970,17 @@
       </c>
       <c r="K8" s="47"/>
       <c r="L8" s="48"/>
-      <c r="M8" s="147"/>
-      <c r="N8" s="148"/>
+      <c r="M8" s="117"/>
+      <c r="N8" s="118"/>
       <c r="O8" s="10"/>
     </row>
     <row r="9" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A9" s="2"/>
-      <c r="B9" s="137"/>
-      <c r="C9" s="128" t="s">
+      <c r="B9" s="138"/>
+      <c r="C9" s="142" t="s">
         <v>27</v>
       </c>
-      <c r="D9" s="129"/>
+      <c r="D9" s="143"/>
       <c r="E9" s="40">
         <v>0.39583333333333331</v>
       </c>
@@ -3005,17 +3005,17 @@
       <c r="L9" s="41">
         <v>0.77083333333333337</v>
       </c>
-      <c r="M9" s="145"/>
-      <c r="N9" s="146"/>
+      <c r="M9" s="125"/>
+      <c r="N9" s="126"/>
       <c r="O9" s="10"/>
     </row>
     <row r="10" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A10" s="2"/>
-      <c r="B10" s="137"/>
-      <c r="C10" s="128" t="s">
+      <c r="B10" s="138"/>
+      <c r="C10" s="142" t="s">
         <v>28</v>
       </c>
-      <c r="D10" s="129"/>
+      <c r="D10" s="143"/>
       <c r="E10" s="45">
         <v>0.36458333333333331</v>
       </c>
@@ -3032,15 +3032,15 @@
       </c>
       <c r="K10" s="47"/>
       <c r="L10" s="48"/>
-      <c r="M10" s="147"/>
-      <c r="N10" s="148"/>
+      <c r="M10" s="117"/>
+      <c r="N10" s="118"/>
       <c r="O10" s="10"/>
     </row>
     <row r="11" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A11" s="2"/>
-      <c r="B11" s="137"/>
-      <c r="C11" s="128"/>
-      <c r="D11" s="129"/>
+      <c r="B11" s="138"/>
+      <c r="C11" s="142"/>
+      <c r="D11" s="143"/>
       <c r="E11" s="40">
         <v>0.66666666666666663</v>
       </c>
@@ -3057,17 +3057,17 @@
       </c>
       <c r="K11" s="40"/>
       <c r="L11" s="41"/>
-      <c r="M11" s="145"/>
-      <c r="N11" s="146"/>
+      <c r="M11" s="125"/>
+      <c r="N11" s="126"/>
       <c r="O11" s="10"/>
     </row>
     <row r="12" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>
-      <c r="B12" s="137"/>
-      <c r="C12" s="134" t="s">
+      <c r="B12" s="138"/>
+      <c r="C12" s="135" t="s">
         <v>29</v>
       </c>
-      <c r="D12" s="135"/>
+      <c r="D12" s="136"/>
       <c r="E12" s="45">
         <v>0.33333333333333331</v>
       </c>
@@ -3084,17 +3084,17 @@
       </c>
       <c r="K12" s="45"/>
       <c r="L12" s="46"/>
-      <c r="M12" s="147" t="s">
+      <c r="M12" s="117" t="s">
         <v>36</v>
       </c>
-      <c r="N12" s="148"/>
+      <c r="N12" s="118"/>
       <c r="O12" s="10"/>
     </row>
     <row r="13" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A13" s="2"/>
-      <c r="B13" s="137"/>
-      <c r="C13" s="134"/>
-      <c r="D13" s="135"/>
+      <c r="B13" s="138"/>
+      <c r="C13" s="135"/>
+      <c r="D13" s="136"/>
       <c r="E13" s="40">
         <v>0.45833333333333331</v>
       </c>
@@ -3111,15 +3111,15 @@
       </c>
       <c r="K13" s="40"/>
       <c r="L13" s="41"/>
-      <c r="M13" s="145"/>
-      <c r="N13" s="146"/>
+      <c r="M13" s="125"/>
+      <c r="N13" s="126"/>
       <c r="O13" s="10"/>
     </row>
     <row r="14" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A14" s="2"/>
-      <c r="B14" s="137"/>
-      <c r="C14" s="134"/>
-      <c r="D14" s="135"/>
+      <c r="B14" s="138"/>
+      <c r="C14" s="135"/>
+      <c r="D14" s="136"/>
       <c r="E14" s="45"/>
       <c r="F14" s="46"/>
       <c r="G14" s="45">
@@ -3136,15 +3136,15 @@
       <c r="L14" s="46">
         <v>0.72916666666666663</v>
       </c>
-      <c r="M14" s="147"/>
-      <c r="N14" s="148"/>
+      <c r="M14" s="117"/>
+      <c r="N14" s="118"/>
       <c r="O14" s="10"/>
     </row>
     <row r="15" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A15" s="2"/>
-      <c r="B15" s="137"/>
-      <c r="C15" s="134"/>
-      <c r="D15" s="135"/>
+      <c r="B15" s="138"/>
+      <c r="C15" s="135"/>
+      <c r="D15" s="136"/>
       <c r="E15" s="40"/>
       <c r="F15" s="41"/>
       <c r="G15" s="40">
@@ -3161,19 +3161,19 @@
       <c r="L15" s="41">
         <v>0.77083333333333337</v>
       </c>
-      <c r="M15" s="145"/>
-      <c r="N15" s="146"/>
+      <c r="M15" s="125"/>
+      <c r="N15" s="126"/>
       <c r="O15" s="10"/>
     </row>
     <row r="16" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
-      <c r="B16" s="130" t="s">
+      <c r="B16" s="139" t="s">
         <v>31</v>
       </c>
-      <c r="C16" s="124" t="s">
+      <c r="C16" s="144" t="s">
         <v>27</v>
       </c>
-      <c r="D16" s="125"/>
+      <c r="D16" s="133"/>
       <c r="E16" s="8"/>
       <c r="F16" s="9"/>
       <c r="G16" s="8">
@@ -3190,15 +3190,15 @@
       <c r="L16" s="9">
         <v>0.42708333333333331</v>
       </c>
-      <c r="M16" s="153"/>
-      <c r="N16" s="154"/>
+      <c r="M16" s="123"/>
+      <c r="N16" s="124"/>
       <c r="O16" s="10"/>
     </row>
     <row r="17" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A17" s="2"/>
-      <c r="B17" s="130"/>
-      <c r="C17" s="124"/>
-      <c r="D17" s="125"/>
+      <c r="B17" s="139"/>
+      <c r="C17" s="144"/>
+      <c r="D17" s="133"/>
       <c r="E17" s="8"/>
       <c r="F17" s="9"/>
       <c r="G17" s="8">
@@ -3215,17 +3215,17 @@
       <c r="L17" s="9">
         <v>0.80208333333333337</v>
       </c>
-      <c r="M17" s="153"/>
-      <c r="N17" s="154"/>
+      <c r="M17" s="123"/>
+      <c r="N17" s="124"/>
       <c r="O17" s="10"/>
     </row>
     <row r="18" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A18" s="2"/>
-      <c r="B18" s="130"/>
-      <c r="C18" s="124" t="s">
+      <c r="B18" s="139"/>
+      <c r="C18" s="144" t="s">
         <v>28</v>
       </c>
-      <c r="D18" s="125"/>
+      <c r="D18" s="133"/>
       <c r="E18" s="8"/>
       <c r="F18" s="9"/>
       <c r="G18" s="8">
@@ -3242,15 +3242,15 @@
       <c r="L18" s="9">
         <v>0.39583333333333331</v>
       </c>
-      <c r="M18" s="153"/>
-      <c r="N18" s="154"/>
+      <c r="M18" s="123"/>
+      <c r="N18" s="124"/>
       <c r="O18" s="10"/>
     </row>
     <row r="19" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A19" s="2"/>
-      <c r="B19" s="130"/>
-      <c r="C19" s="124"/>
-      <c r="D19" s="125"/>
+      <c r="B19" s="139"/>
+      <c r="C19" s="144"/>
+      <c r="D19" s="133"/>
       <c r="E19" s="8"/>
       <c r="F19" s="9"/>
       <c r="G19" s="8">
@@ -3267,17 +3267,17 @@
       <c r="L19" s="9">
         <v>0.69791666666666663</v>
       </c>
-      <c r="M19" s="153"/>
-      <c r="N19" s="154"/>
+      <c r="M19" s="123"/>
+      <c r="N19" s="124"/>
       <c r="O19" s="10"/>
     </row>
     <row r="20" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A20" s="2"/>
-      <c r="B20" s="130"/>
-      <c r="C20" s="126" t="s">
+      <c r="B20" s="139"/>
+      <c r="C20" s="145" t="s">
         <v>29</v>
       </c>
-      <c r="D20" s="127"/>
+      <c r="D20" s="146"/>
       <c r="E20" s="8"/>
       <c r="F20" s="9"/>
       <c r="G20" s="8">
@@ -3294,17 +3294,17 @@
       <c r="L20" s="9">
         <v>0.36458333333333331</v>
       </c>
-      <c r="M20" s="153" t="s">
+      <c r="M20" s="123" t="s">
         <v>37</v>
       </c>
-      <c r="N20" s="154"/>
+      <c r="N20" s="124"/>
       <c r="O20" s="10"/>
     </row>
     <row r="21" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A21" s="2"/>
-      <c r="B21" s="130"/>
-      <c r="C21" s="126"/>
-      <c r="D21" s="127"/>
+      <c r="B21" s="139"/>
+      <c r="C21" s="145"/>
+      <c r="D21" s="146"/>
       <c r="E21" s="8"/>
       <c r="F21" s="9"/>
       <c r="G21" s="8">
@@ -3321,19 +3321,19 @@
       <c r="L21" s="9">
         <v>0.83333333333333337</v>
       </c>
-      <c r="M21" s="153"/>
-      <c r="N21" s="154"/>
+      <c r="M21" s="123"/>
+      <c r="N21" s="124"/>
       <c r="O21" s="10"/>
     </row>
     <row r="22" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A22" s="2"/>
-      <c r="B22" s="137" t="s">
+      <c r="B22" s="138" t="s">
         <v>33</v>
       </c>
-      <c r="C22" s="128" t="s">
+      <c r="C22" s="142" t="s">
         <v>28</v>
       </c>
-      <c r="D22" s="129"/>
+      <c r="D22" s="143"/>
       <c r="E22" s="45">
         <v>0.69791666666666663</v>
       </c>
@@ -3350,17 +3350,17 @@
       </c>
       <c r="K22" s="45"/>
       <c r="L22" s="46"/>
-      <c r="M22" s="147"/>
-      <c r="N22" s="148"/>
+      <c r="M22" s="117"/>
+      <c r="N22" s="118"/>
       <c r="O22" s="10"/>
     </row>
     <row r="23" spans="1:15" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2"/>
-      <c r="B23" s="137"/>
-      <c r="C23" s="128" t="s">
+      <c r="B23" s="138"/>
+      <c r="C23" s="142" t="s">
         <v>29</v>
       </c>
-      <c r="D23" s="129"/>
+      <c r="D23" s="143"/>
       <c r="E23" s="45">
         <v>0.80208333333333337</v>
       </c>
@@ -3377,52 +3377,52 @@
       </c>
       <c r="K23" s="45"/>
       <c r="L23" s="46"/>
-      <c r="M23" s="147"/>
-      <c r="N23" s="148"/>
+      <c r="M23" s="117"/>
+      <c r="N23" s="118"/>
       <c r="O23" s="10"/>
     </row>
     <row r="24" spans="1:15" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2"/>
-      <c r="B24" s="130" t="s">
+      <c r="B24" s="139" t="s">
         <v>30</v>
       </c>
-      <c r="C24" s="126"/>
-      <c r="D24" s="127"/>
-      <c r="E24" s="138">
+      <c r="C24" s="145"/>
+      <c r="D24" s="146"/>
+      <c r="E24" s="127">
         <v>0.5</v>
       </c>
-      <c r="F24" s="122">
+      <c r="F24" s="129">
         <v>0.53125</v>
       </c>
-      <c r="G24" s="138"/>
-      <c r="H24" s="122"/>
-      <c r="I24" s="142">
+      <c r="G24" s="127"/>
+      <c r="H24" s="129"/>
+      <c r="I24" s="131">
         <v>0.5</v>
       </c>
-      <c r="J24" s="125">
+      <c r="J24" s="133">
         <v>0.53125</v>
       </c>
-      <c r="K24" s="138"/>
-      <c r="L24" s="125"/>
-      <c r="M24" s="149"/>
-      <c r="N24" s="150"/>
+      <c r="K24" s="127"/>
+      <c r="L24" s="133"/>
+      <c r="M24" s="119"/>
+      <c r="N24" s="120"/>
       <c r="O24" s="10"/>
     </row>
     <row r="25" spans="1:15" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="2"/>
-      <c r="B25" s="131"/>
-      <c r="C25" s="132"/>
-      <c r="D25" s="133"/>
-      <c r="E25" s="139"/>
-      <c r="F25" s="123"/>
-      <c r="G25" s="139"/>
-      <c r="H25" s="123"/>
-      <c r="I25" s="143"/>
-      <c r="J25" s="144"/>
-      <c r="K25" s="139"/>
-      <c r="L25" s="144"/>
-      <c r="M25" s="151"/>
-      <c r="N25" s="152"/>
+      <c r="B25" s="147"/>
+      <c r="C25" s="148"/>
+      <c r="D25" s="149"/>
+      <c r="E25" s="128"/>
+      <c r="F25" s="130"/>
+      <c r="G25" s="128"/>
+      <c r="H25" s="130"/>
+      <c r="I25" s="132"/>
+      <c r="J25" s="134"/>
+      <c r="K25" s="128"/>
+      <c r="L25" s="134"/>
+      <c r="M25" s="121"/>
+      <c r="N25" s="122"/>
       <c r="O25" s="10"/>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
@@ -3463,15 +3463,35 @@
     </row>
   </sheetData>
   <mergeCells count="49">
-    <mergeCell ref="M22:N22"/>
-    <mergeCell ref="M23:N23"/>
-    <mergeCell ref="M24:N25"/>
-    <mergeCell ref="M16:N16"/>
-    <mergeCell ref="M17:N17"/>
-    <mergeCell ref="M18:N18"/>
-    <mergeCell ref="M19:N19"/>
-    <mergeCell ref="M20:N20"/>
-    <mergeCell ref="M21:N21"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="F24:F25"/>
+    <mergeCell ref="C16:D17"/>
+    <mergeCell ref="C18:D19"/>
+    <mergeCell ref="C20:D21"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="B24:D25"/>
+    <mergeCell ref="C12:D15"/>
+    <mergeCell ref="B5:B15"/>
+    <mergeCell ref="B16:B21"/>
+    <mergeCell ref="B22:B23"/>
+    <mergeCell ref="E24:E25"/>
+    <mergeCell ref="C5:D6"/>
+    <mergeCell ref="C7:D8"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="C10:D11"/>
+    <mergeCell ref="G24:G25"/>
+    <mergeCell ref="H24:H25"/>
+    <mergeCell ref="I24:I25"/>
+    <mergeCell ref="L24:L25"/>
+    <mergeCell ref="J24:J25"/>
+    <mergeCell ref="K24:K25"/>
     <mergeCell ref="M15:N15"/>
     <mergeCell ref="M5:N5"/>
     <mergeCell ref="M6:N6"/>
@@ -3483,35 +3503,15 @@
     <mergeCell ref="M12:N12"/>
     <mergeCell ref="M13:N13"/>
     <mergeCell ref="M14:N14"/>
-    <mergeCell ref="G24:G25"/>
-    <mergeCell ref="H24:H25"/>
-    <mergeCell ref="I24:I25"/>
-    <mergeCell ref="L24:L25"/>
-    <mergeCell ref="J24:J25"/>
-    <mergeCell ref="K24:K25"/>
-    <mergeCell ref="C12:D15"/>
-    <mergeCell ref="B5:B15"/>
-    <mergeCell ref="B16:B21"/>
-    <mergeCell ref="B22:B23"/>
-    <mergeCell ref="E24:E25"/>
-    <mergeCell ref="C5:D6"/>
-    <mergeCell ref="C7:D8"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="C10:D11"/>
-    <mergeCell ref="F24:F25"/>
-    <mergeCell ref="C16:D17"/>
-    <mergeCell ref="C18:D19"/>
-    <mergeCell ref="C20:D21"/>
-    <mergeCell ref="C22:D22"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="B24:D25"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="E4:F4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="M4:N4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="M22:N22"/>
+    <mergeCell ref="M23:N23"/>
+    <mergeCell ref="M24:N25"/>
+    <mergeCell ref="M16:N16"/>
+    <mergeCell ref="M17:N17"/>
+    <mergeCell ref="M18:N18"/>
+    <mergeCell ref="M19:N19"/>
+    <mergeCell ref="M20:N20"/>
+    <mergeCell ref="M21:N21"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
@@ -3584,23 +3584,23 @@
       <c r="D3" s="157" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="119"/>
-      <c r="F3" s="118" t="s">
+      <c r="E3" s="152"/>
+      <c r="F3" s="151" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="119"/>
-      <c r="H3" s="118" t="s">
+      <c r="G3" s="152"/>
+      <c r="H3" s="151" t="s">
         <v>4</v>
       </c>
-      <c r="I3" s="119"/>
-      <c r="J3" s="118" t="s">
+      <c r="I3" s="152"/>
+      <c r="J3" s="151" t="s">
         <v>5</v>
       </c>
-      <c r="K3" s="119"/>
-      <c r="L3" s="118" t="s">
+      <c r="K3" s="152"/>
+      <c r="L3" s="151" t="s">
         <v>6</v>
       </c>
-      <c r="M3" s="119"/>
+      <c r="M3" s="152"/>
       <c r="N3" s="2"/>
     </row>
     <row r="4" spans="1:14" ht="18.75" x14ac:dyDescent="0.25">
@@ -4115,10 +4115,10 @@
       <c r="E4" s="65" t="s">
         <v>68</v>
       </c>
-      <c r="F4" s="170" t="s">
+      <c r="F4" s="179" t="s">
         <v>69</v>
       </c>
-      <c r="G4" s="170"/>
+      <c r="G4" s="179"/>
       <c r="H4" s="66" t="s">
         <v>73</v>
       </c>
@@ -4129,10 +4129,10 @@
     </row>
     <row r="5" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A5" s="2"/>
-      <c r="B5" s="189" t="s">
+      <c r="B5" s="164" t="s">
         <v>66</v>
       </c>
-      <c r="C5" s="142" t="s">
+      <c r="C5" s="131" t="s">
         <v>40</v>
       </c>
       <c r="D5" s="16" t="s">
@@ -4147,18 +4147,18 @@
       <c r="G5" s="16">
         <v>0.39583333333333331</v>
       </c>
-      <c r="H5" s="178">
+      <c r="H5" s="187">
         <v>10</v>
       </c>
-      <c r="I5" s="125" t="s">
+      <c r="I5" s="133" t="s">
         <v>90</v>
       </c>
       <c r="J5" s="2"/>
     </row>
     <row r="6" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2"/>
-      <c r="B6" s="189"/>
-      <c r="C6" s="143"/>
+      <c r="B6" s="164"/>
+      <c r="C6" s="132"/>
       <c r="D6" s="67" t="s">
         <v>46</v>
       </c>
@@ -4171,14 +4171,14 @@
       <c r="G6" s="67">
         <v>0.75</v>
       </c>
-      <c r="H6" s="179"/>
-      <c r="I6" s="144"/>
+      <c r="H6" s="188"/>
+      <c r="I6" s="134"/>
       <c r="J6" s="2"/>
     </row>
     <row r="7" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
-      <c r="B7" s="189"/>
-      <c r="C7" s="191" t="s">
+      <c r="B7" s="164"/>
+      <c r="C7" s="166" t="s">
         <v>43</v>
       </c>
       <c r="D7" s="72" t="s">
@@ -4193,18 +4193,18 @@
       <c r="G7" s="69">
         <v>0.41666666666666669</v>
       </c>
-      <c r="H7" s="174">
+      <c r="H7" s="183">
         <v>16</v>
       </c>
-      <c r="I7" s="171" t="s">
+      <c r="I7" s="180" t="s">
         <v>91</v>
       </c>
       <c r="J7" s="2"/>
     </row>
     <row r="8" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A8" s="2"/>
-      <c r="B8" s="189"/>
-      <c r="C8" s="192"/>
+      <c r="B8" s="164"/>
+      <c r="C8" s="167"/>
       <c r="D8" s="23" t="s">
         <v>48</v>
       </c>
@@ -4217,14 +4217,14 @@
       <c r="G8" s="60">
         <v>0.76041666666666663</v>
       </c>
-      <c r="H8" s="175"/>
-      <c r="I8" s="167"/>
+      <c r="H8" s="184"/>
+      <c r="I8" s="176"/>
       <c r="J8" s="10"/>
     </row>
     <row r="9" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A9" s="2"/>
-      <c r="B9" s="189"/>
-      <c r="C9" s="192"/>
+      <c r="B9" s="164"/>
+      <c r="C9" s="167"/>
       <c r="D9" s="23" t="s">
         <v>49</v>
       </c>
@@ -4237,28 +4237,28 @@
       <c r="G9" s="60">
         <v>0.79166666666666663</v>
       </c>
-      <c r="H9" s="175"/>
-      <c r="I9" s="167" t="s">
+      <c r="H9" s="184"/>
+      <c r="I9" s="176" t="s">
         <v>92</v>
       </c>
       <c r="J9" s="10"/>
     </row>
     <row r="10" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2"/>
-      <c r="B10" s="189"/>
-      <c r="C10" s="193"/>
+      <c r="B10" s="164"/>
+      <c r="C10" s="168"/>
       <c r="D10" s="30"/>
       <c r="E10" s="71"/>
       <c r="F10" s="71"/>
       <c r="G10" s="71"/>
-      <c r="H10" s="176"/>
-      <c r="I10" s="168"/>
+      <c r="H10" s="185"/>
+      <c r="I10" s="177"/>
       <c r="J10" s="10"/>
     </row>
     <row r="11" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A11" s="2"/>
-      <c r="B11" s="189"/>
-      <c r="C11" s="194" t="s">
+      <c r="B11" s="164"/>
+      <c r="C11" s="169" t="s">
         <v>71</v>
       </c>
       <c r="D11" s="75" t="s">
@@ -4273,7 +4273,7 @@
       <c r="G11" s="76">
         <v>0.45833333333333331</v>
       </c>
-      <c r="H11" s="180">
+      <c r="H11" s="189">
         <v>14</v>
       </c>
       <c r="I11" s="77" t="s">
@@ -4283,8 +4283,8 @@
     </row>
     <row r="12" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>
-      <c r="B12" s="189"/>
-      <c r="C12" s="195"/>
+      <c r="B12" s="164"/>
+      <c r="C12" s="170"/>
       <c r="D12" s="78" t="s">
         <v>74</v>
       </c>
@@ -4297,7 +4297,7 @@
       <c r="G12" s="61">
         <v>0.45833333333333331</v>
       </c>
-      <c r="H12" s="181"/>
+      <c r="H12" s="190"/>
       <c r="I12" s="57" t="s">
         <v>91</v>
       </c>
@@ -4305,8 +4305,8 @@
     </row>
     <row r="13" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A13" s="2"/>
-      <c r="B13" s="189"/>
-      <c r="C13" s="195"/>
+      <c r="B13" s="164"/>
+      <c r="C13" s="170"/>
       <c r="D13" s="78" t="s">
         <v>74</v>
       </c>
@@ -4319,16 +4319,16 @@
       <c r="G13" s="61">
         <v>0.77083333333333337</v>
       </c>
-      <c r="H13" s="181"/>
-      <c r="I13" s="172" t="s">
+      <c r="H13" s="190"/>
+      <c r="I13" s="181" t="s">
         <v>93</v>
       </c>
       <c r="J13" s="10"/>
     </row>
     <row r="14" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A14" s="2"/>
-      <c r="B14" s="189"/>
-      <c r="C14" s="195"/>
+      <c r="B14" s="164"/>
+      <c r="C14" s="170"/>
       <c r="D14" s="78" t="s">
         <v>75</v>
       </c>
@@ -4341,14 +4341,14 @@
       <c r="G14" s="61">
         <v>0.45833333333333331</v>
       </c>
-      <c r="H14" s="181"/>
-      <c r="I14" s="172"/>
+      <c r="H14" s="190"/>
+      <c r="I14" s="181"/>
       <c r="J14" s="10"/>
     </row>
     <row r="15" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A15" s="2"/>
-      <c r="B15" s="189"/>
-      <c r="C15" s="195"/>
+      <c r="B15" s="164"/>
+      <c r="C15" s="170"/>
       <c r="D15" s="78" t="s">
         <v>75</v>
       </c>
@@ -4361,14 +4361,14 @@
       <c r="G15" s="61">
         <v>0.80208333333333337</v>
       </c>
-      <c r="H15" s="181"/>
-      <c r="I15" s="172"/>
+      <c r="H15" s="190"/>
+      <c r="I15" s="181"/>
       <c r="J15" s="10"/>
     </row>
     <row r="16" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
-      <c r="B16" s="189"/>
-      <c r="C16" s="195"/>
+      <c r="B16" s="164"/>
+      <c r="C16" s="170"/>
       <c r="D16" s="78" t="s">
         <v>76</v>
       </c>
@@ -4381,14 +4381,14 @@
       <c r="G16" s="61">
         <v>0.42708333333333331</v>
       </c>
-      <c r="H16" s="181"/>
-      <c r="I16" s="172"/>
+      <c r="H16" s="190"/>
+      <c r="I16" s="181"/>
       <c r="J16" s="10"/>
     </row>
     <row r="17" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A17" s="2"/>
-      <c r="B17" s="189"/>
-      <c r="C17" s="195"/>
+      <c r="B17" s="164"/>
+      <c r="C17" s="170"/>
       <c r="D17" s="78" t="s">
         <v>76</v>
       </c>
@@ -4401,14 +4401,14 @@
       <c r="G17" s="61">
         <v>0.77083333333333337</v>
       </c>
-      <c r="H17" s="181"/>
-      <c r="I17" s="172"/>
+      <c r="H17" s="190"/>
+      <c r="I17" s="181"/>
       <c r="J17" s="10"/>
     </row>
     <row r="18" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A18" s="2"/>
-      <c r="B18" s="189"/>
-      <c r="C18" s="195"/>
+      <c r="B18" s="164"/>
+      <c r="C18" s="170"/>
       <c r="D18" s="78" t="s">
         <v>77</v>
       </c>
@@ -4421,14 +4421,14 @@
       <c r="G18" s="61">
         <v>0.39583333333333331</v>
       </c>
-      <c r="H18" s="181"/>
-      <c r="I18" s="172"/>
+      <c r="H18" s="190"/>
+      <c r="I18" s="181"/>
       <c r="J18" s="10"/>
     </row>
     <row r="19" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2"/>
-      <c r="B19" s="189"/>
-      <c r="C19" s="195"/>
+      <c r="B19" s="164"/>
+      <c r="C19" s="170"/>
       <c r="D19" s="79" t="s">
         <v>77</v>
       </c>
@@ -4441,14 +4441,14 @@
       <c r="G19" s="80">
         <v>0.69791666666666663</v>
       </c>
-      <c r="H19" s="182"/>
-      <c r="I19" s="173"/>
+      <c r="H19" s="191"/>
+      <c r="I19" s="182"/>
       <c r="J19" s="10"/>
     </row>
     <row r="20" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A20" s="2"/>
-      <c r="B20" s="189"/>
-      <c r="C20" s="195"/>
+      <c r="B20" s="164"/>
+      <c r="C20" s="170"/>
       <c r="D20" s="81" t="s">
         <v>78</v>
       </c>
@@ -4461,7 +4461,7 @@
       <c r="G20" s="82">
         <v>0.36458333333333331</v>
       </c>
-      <c r="H20" s="183">
+      <c r="H20" s="192">
         <v>12</v>
       </c>
       <c r="I20" s="83" t="s">
@@ -4471,8 +4471,8 @@
     </row>
     <row r="21" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A21" s="2"/>
-      <c r="B21" s="189"/>
-      <c r="C21" s="195"/>
+      <c r="B21" s="164"/>
+      <c r="C21" s="170"/>
       <c r="D21" s="84" t="s">
         <v>78</v>
       </c>
@@ -4485,7 +4485,7 @@
       <c r="G21" s="62">
         <v>0.48958333333333331</v>
       </c>
-      <c r="H21" s="184"/>
+      <c r="H21" s="193"/>
       <c r="I21" s="58" t="s">
         <v>94</v>
       </c>
@@ -4493,8 +4493,8 @@
     </row>
     <row r="22" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A22" s="2"/>
-      <c r="B22" s="189"/>
-      <c r="C22" s="195"/>
+      <c r="B22" s="164"/>
+      <c r="C22" s="170"/>
       <c r="D22" s="84" t="s">
         <v>78</v>
       </c>
@@ -4507,7 +4507,7 @@
       <c r="G22" s="62">
         <v>0.72916666666666663</v>
       </c>
-      <c r="H22" s="184"/>
+      <c r="H22" s="193"/>
       <c r="I22" s="58" t="s">
         <v>93</v>
       </c>
@@ -4515,8 +4515,8 @@
     </row>
     <row r="23" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A23" s="2"/>
-      <c r="B23" s="189"/>
-      <c r="C23" s="195"/>
+      <c r="B23" s="164"/>
+      <c r="C23" s="170"/>
       <c r="D23" s="84" t="s">
         <v>78</v>
       </c>
@@ -4529,7 +4529,7 @@
       <c r="G23" s="62">
         <v>0.77083333333333337</v>
       </c>
-      <c r="H23" s="184"/>
+      <c r="H23" s="193"/>
       <c r="I23" s="58" t="s">
         <v>92</v>
       </c>
@@ -4537,8 +4537,8 @@
     </row>
     <row r="24" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="2"/>
-      <c r="B24" s="189"/>
-      <c r="C24" s="195"/>
+      <c r="B24" s="164"/>
+      <c r="C24" s="170"/>
       <c r="D24" s="85" t="s">
         <v>78</v>
       </c>
@@ -4551,7 +4551,7 @@
       <c r="G24" s="86">
         <v>0.46875</v>
       </c>
-      <c r="H24" s="185"/>
+      <c r="H24" s="194"/>
       <c r="I24" s="87" t="s">
         <v>94</v>
       </c>
@@ -4559,8 +4559,8 @@
     </row>
     <row r="25" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A25" s="2"/>
-      <c r="B25" s="189"/>
-      <c r="C25" s="195"/>
+      <c r="B25" s="164"/>
+      <c r="C25" s="170"/>
       <c r="D25" s="88" t="s">
         <v>79</v>
       </c>
@@ -4573,18 +4573,18 @@
       <c r="G25" s="89">
         <v>0.42708333333333331</v>
       </c>
-      <c r="H25" s="186">
+      <c r="H25" s="195">
         <v>14</v>
       </c>
-      <c r="I25" s="164" t="s">
+      <c r="I25" s="173" t="s">
         <v>93</v>
       </c>
       <c r="J25" s="10"/>
     </row>
     <row r="26" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A26" s="2"/>
-      <c r="B26" s="189"/>
-      <c r="C26" s="195"/>
+      <c r="B26" s="164"/>
+      <c r="C26" s="170"/>
       <c r="D26" s="90" t="s">
         <v>79</v>
       </c>
@@ -4597,14 +4597,14 @@
       <c r="G26" s="63">
         <v>0.80208333333333337</v>
       </c>
-      <c r="H26" s="187"/>
-      <c r="I26" s="165"/>
+      <c r="H26" s="196"/>
+      <c r="I26" s="174"/>
       <c r="J26" s="10"/>
     </row>
     <row r="27" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A27" s="2"/>
-      <c r="B27" s="189"/>
-      <c r="C27" s="195"/>
+      <c r="B27" s="164"/>
+      <c r="C27" s="170"/>
       <c r="D27" s="90" t="s">
         <v>80</v>
       </c>
@@ -4617,14 +4617,14 @@
       <c r="G27" s="63">
         <v>0.39583333333333331</v>
       </c>
-      <c r="H27" s="187"/>
-      <c r="I27" s="165"/>
+      <c r="H27" s="196"/>
+      <c r="I27" s="174"/>
       <c r="J27" s="10"/>
     </row>
     <row r="28" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="2"/>
-      <c r="B28" s="189"/>
-      <c r="C28" s="195"/>
+      <c r="B28" s="164"/>
+      <c r="C28" s="170"/>
       <c r="D28" s="91" t="s">
         <v>80</v>
       </c>
@@ -4637,14 +4637,14 @@
       <c r="G28" s="92">
         <v>0.69791666666666663</v>
       </c>
-      <c r="H28" s="188"/>
-      <c r="I28" s="166"/>
+      <c r="H28" s="197"/>
+      <c r="I28" s="175"/>
       <c r="J28" s="10"/>
     </row>
     <row r="29" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A29" s="2"/>
-      <c r="B29" s="189"/>
-      <c r="C29" s="195"/>
+      <c r="B29" s="164"/>
+      <c r="C29" s="170"/>
       <c r="D29" s="93" t="s">
         <v>81</v>
       </c>
@@ -4657,7 +4657,7 @@
       <c r="G29" s="69">
         <v>0.36458333333333331</v>
       </c>
-      <c r="H29" s="174">
+      <c r="H29" s="183">
         <v>12</v>
       </c>
       <c r="I29" s="94" t="s">
@@ -4667,8 +4667,8 @@
     </row>
     <row r="30" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A30" s="2"/>
-      <c r="B30" s="189"/>
-      <c r="C30" s="195"/>
+      <c r="B30" s="164"/>
+      <c r="C30" s="170"/>
       <c r="D30" s="25" t="s">
         <v>81</v>
       </c>
@@ -4681,16 +4681,16 @@
       <c r="G30" s="60">
         <v>0.83333333333333337</v>
       </c>
-      <c r="H30" s="175"/>
-      <c r="I30" s="167" t="s">
+      <c r="H30" s="184"/>
+      <c r="I30" s="176" t="s">
         <v>94</v>
       </c>
       <c r="J30" s="10"/>
     </row>
     <row r="31" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="2"/>
-      <c r="B31" s="189"/>
-      <c r="C31" s="195"/>
+      <c r="B31" s="164"/>
+      <c r="C31" s="170"/>
       <c r="D31" s="33" t="s">
         <v>81</v>
       </c>
@@ -4703,14 +4703,14 @@
       <c r="G31" s="70">
         <v>0.41666666666666669</v>
       </c>
-      <c r="H31" s="176"/>
-      <c r="I31" s="168"/>
+      <c r="H31" s="185"/>
+      <c r="I31" s="177"/>
       <c r="J31" s="10"/>
     </row>
     <row r="32" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A32" s="2"/>
-      <c r="B32" s="189"/>
-      <c r="C32" s="195"/>
+      <c r="B32" s="164"/>
+      <c r="C32" s="170"/>
       <c r="D32" s="75" t="s">
         <v>83</v>
       </c>
@@ -4733,8 +4733,8 @@
     </row>
     <row r="33" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A33" s="2"/>
-      <c r="B33" s="189"/>
-      <c r="C33" s="195"/>
+      <c r="B33" s="164"/>
+      <c r="C33" s="170"/>
       <c r="D33" s="84" t="s">
         <v>84</v>
       </c>
@@ -4757,8 +4757,8 @@
     </row>
     <row r="34" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="2"/>
-      <c r="B34" s="189"/>
-      <c r="C34" s="196"/>
+      <c r="B34" s="164"/>
+      <c r="C34" s="171"/>
       <c r="D34" s="79" t="s">
         <v>82</v>
       </c>
@@ -4781,8 +4781,8 @@
     </row>
     <row r="35" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A35" s="2"/>
-      <c r="B35" s="189"/>
-      <c r="C35" s="197" t="s">
+      <c r="B35" s="164"/>
+      <c r="C35" s="172" t="s">
         <v>44</v>
       </c>
       <c r="D35" s="99" t="s">
@@ -4797,7 +4797,7 @@
       <c r="G35" s="69">
         <v>0.77083333333333337</v>
       </c>
-      <c r="H35" s="174">
+      <c r="H35" s="183">
         <v>20</v>
       </c>
       <c r="I35" s="100" t="s">
@@ -4807,7 +4807,7 @@
     </row>
     <row r="36" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A36" s="2"/>
-      <c r="B36" s="189"/>
+      <c r="B36" s="164"/>
       <c r="C36" s="155"/>
       <c r="D36" s="27" t="s">
         <v>48</v>
@@ -4821,7 +4821,7 @@
       <c r="G36" s="60">
         <v>0.78472222222222221</v>
       </c>
-      <c r="H36" s="175"/>
+      <c r="H36" s="184"/>
       <c r="I36" s="24" t="s">
         <v>94</v>
       </c>
@@ -4829,7 +4829,7 @@
     </row>
     <row r="37" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A37" s="2"/>
-      <c r="B37" s="189"/>
+      <c r="B37" s="164"/>
       <c r="C37" s="155"/>
       <c r="D37" s="27" t="s">
         <v>49</v>
@@ -4843,7 +4843,7 @@
       <c r="G37" s="60">
         <v>0.80555555555555558</v>
       </c>
-      <c r="H37" s="175"/>
+      <c r="H37" s="184"/>
       <c r="I37" s="24" t="s">
         <v>91</v>
       </c>
@@ -4851,7 +4851,7 @@
     </row>
     <row r="38" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A38" s="2"/>
-      <c r="B38" s="189"/>
+      <c r="B38" s="164"/>
       <c r="C38" s="155"/>
       <c r="D38" s="27" t="s">
         <v>49</v>
@@ -4865,7 +4865,7 @@
       <c r="G38" s="60">
         <v>0.81944444444444442</v>
       </c>
-      <c r="H38" s="175"/>
+      <c r="H38" s="184"/>
       <c r="I38" s="24" t="s">
         <v>94</v>
       </c>
@@ -4873,7 +4873,7 @@
     </row>
     <row r="39" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A39" s="2"/>
-      <c r="B39" s="189"/>
+      <c r="B39" s="164"/>
       <c r="C39" s="155"/>
       <c r="D39" s="27" t="s">
         <v>50</v>
@@ -4887,7 +4887,7 @@
       <c r="G39" s="60">
         <v>0.84027777777777779</v>
       </c>
-      <c r="H39" s="175"/>
+      <c r="H39" s="184"/>
       <c r="I39" s="24" t="s">
         <v>91</v>
       </c>
@@ -4895,7 +4895,7 @@
     </row>
     <row r="40" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A40" s="2"/>
-      <c r="B40" s="189"/>
+      <c r="B40" s="164"/>
       <c r="C40" s="155"/>
       <c r="D40" s="27" t="s">
         <v>50</v>
@@ -4909,7 +4909,7 @@
       <c r="G40" s="60">
         <v>0.85416666666666663</v>
       </c>
-      <c r="H40" s="175"/>
+      <c r="H40" s="184"/>
       <c r="I40" s="24" t="s">
         <v>94</v>
       </c>
@@ -4917,7 +4917,7 @@
     </row>
     <row r="41" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="2"/>
-      <c r="B41" s="189"/>
+      <c r="B41" s="164"/>
       <c r="C41" s="156"/>
       <c r="D41" s="32" t="s">
         <v>51</v>
@@ -4931,7 +4931,7 @@
       <c r="G41" s="70">
         <v>0.72222222222222221</v>
       </c>
-      <c r="H41" s="176"/>
+      <c r="H41" s="185"/>
       <c r="I41" s="31" t="s">
         <v>91</v>
       </c>
@@ -4939,8 +4939,8 @@
     </row>
     <row r="42" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A42" s="2"/>
-      <c r="B42" s="189"/>
-      <c r="C42" s="194" t="s">
+      <c r="B42" s="164"/>
+      <c r="C42" s="169" t="s">
         <v>72</v>
       </c>
       <c r="D42" s="101" t="s">
@@ -4955,18 +4955,18 @@
       <c r="G42" s="102">
         <v>0.44444444444444442</v>
       </c>
-      <c r="H42" s="177">
+      <c r="H42" s="186">
         <v>12</v>
       </c>
-      <c r="I42" s="169" t="s">
+      <c r="I42" s="178" t="s">
         <v>94</v>
       </c>
       <c r="J42" s="10"/>
     </row>
     <row r="43" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A43" s="2"/>
-      <c r="B43" s="189"/>
-      <c r="C43" s="195"/>
+      <c r="B43" s="164"/>
+      <c r="C43" s="170"/>
       <c r="D43" s="15" t="s">
         <v>48</v>
       </c>
@@ -4979,14 +4979,14 @@
       <c r="G43" s="16">
         <v>0.44444444444444442</v>
       </c>
-      <c r="H43" s="178"/>
-      <c r="I43" s="125"/>
+      <c r="H43" s="187"/>
+      <c r="I43" s="133"/>
       <c r="J43" s="10"/>
     </row>
     <row r="44" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A44" s="2"/>
-      <c r="B44" s="189"/>
-      <c r="C44" s="195"/>
+      <c r="B44" s="164"/>
+      <c r="C44" s="170"/>
       <c r="D44" s="15" t="s">
         <v>49</v>
       </c>
@@ -4999,14 +4999,14 @@
       <c r="G44" s="16">
         <v>0.40972222222222221</v>
       </c>
-      <c r="H44" s="178"/>
-      <c r="I44" s="125"/>
+      <c r="H44" s="187"/>
+      <c r="I44" s="133"/>
       <c r="J44" s="10"/>
     </row>
     <row r="45" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="2"/>
-      <c r="B45" s="189"/>
-      <c r="C45" s="196"/>
+      <c r="B45" s="164"/>
+      <c r="C45" s="171"/>
       <c r="D45" s="17" t="s">
         <v>49</v>
       </c>
@@ -5019,13 +5019,13 @@
       <c r="G45" s="67">
         <v>0.70138888888888884</v>
       </c>
-      <c r="H45" s="179"/>
-      <c r="I45" s="144"/>
+      <c r="H45" s="188"/>
+      <c r="I45" s="134"/>
       <c r="J45" s="10"/>
     </row>
     <row r="46" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="2"/>
-      <c r="B46" s="189"/>
+      <c r="B46" s="164"/>
       <c r="C46" s="73" t="s">
         <v>42</v>
       </c>
@@ -5051,7 +5051,7 @@
     </row>
     <row r="47" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="2"/>
-      <c r="B47" s="190"/>
+      <c r="B47" s="165"/>
       <c r="C47" s="74" t="s">
         <v>41</v>
       </c>
@@ -5089,12 +5089,6 @@
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="B5:B47"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="C7:C10"/>
-    <mergeCell ref="C11:C34"/>
-    <mergeCell ref="C35:C41"/>
-    <mergeCell ref="C42:C45"/>
     <mergeCell ref="I25:I28"/>
     <mergeCell ref="I30:I31"/>
     <mergeCell ref="I42:I45"/>
@@ -5111,6 +5105,12 @@
     <mergeCell ref="H20:H24"/>
     <mergeCell ref="H25:H28"/>
     <mergeCell ref="H29:H31"/>
+    <mergeCell ref="B5:B47"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="C7:C10"/>
+    <mergeCell ref="C11:C34"/>
+    <mergeCell ref="C35:C41"/>
+    <mergeCell ref="C42:C45"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
@@ -5596,7 +5596,7 @@
         <v>DOM</v>
       </c>
       <c r="B23" s="112">
-        <v>0.66666666666666696</v>
+        <v>0.70833333333333337</v>
       </c>
       <c r="C23" s="112">
         <v>0.90625</v>
@@ -5617,7 +5617,7 @@
         <v>DOM</v>
       </c>
       <c r="B24" s="112">
-        <v>0.66666666666666696</v>
+        <v>0.70833333333333337</v>
       </c>
       <c r="C24" s="112">
         <v>0.90625</v>
@@ -5638,7 +5638,7 @@
         <v>DOM</v>
       </c>
       <c r="B25" s="112">
-        <v>0.66666666666666696</v>
+        <v>0.70833333333333337</v>
       </c>
       <c r="C25" s="112">
         <v>0.90625</v>
@@ -5659,7 +5659,7 @@
         <v>DOM</v>
       </c>
       <c r="B26" s="112">
-        <v>0.66666666666666696</v>
+        <v>0.70833333333333337</v>
       </c>
       <c r="C26" s="112">
         <v>0.90625</v>
@@ -5680,7 +5680,7 @@
         <v>DOM</v>
       </c>
       <c r="B27" s="112">
-        <v>0.66666666666666696</v>
+        <v>0.70833333333333337</v>
       </c>
       <c r="C27" s="112">
         <v>0.90625</v>

</xml_diff>

<commit_message>
Clean Pylance diagnostics and harden optional UI typing paths
Resolve the remaining Pylance issues in clubal.py by hardening optional Tkinter and Pillow code paths, guarding nullable widget ids, normalizing image handling, and simplifying typed refresh/update flows. This keeps runtime behavior unchanged while making the codebase cleaner, safer to maintain, and easier to continue modularizing in Phase 2.
</commit_message>
<xml_diff>
--- a/grade.xlsx
+++ b/grade.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrativo\Documents\GitHub\clubal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{532C5FBE-C8CC-4EDA-AC74-96C05184073D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED0E4B92-89E5-460A-83BE-4B30D3100641}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1499,40 +1499,19 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="20" fontId="5" fillId="9" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="9" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="2" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="8" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="8" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="2" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="20" fontId="5" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1541,16 +1520,34 @@
     <xf numFmtId="20" fontId="5" fillId="2" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="20" fontId="5" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="20" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="20" fontId="5" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="20" fontId="5" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="9" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1565,8 +1562,11 @@
     <xf numFmtId="0" fontId="5" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="20" fontId="5" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="2" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="20" fontId="5" fillId="9" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1574,43 +1574,43 @@
     <xf numFmtId="20" fontId="5" fillId="9" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="20" fontId="5" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="9" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="20" fontId="5" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="8" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="8" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="9" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="9" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="2" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1640,6 +1640,81 @@
     <xf numFmtId="0" fontId="5" fillId="9" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="7" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
@@ -1665,81 +1740,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="7" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2834,7 +2834,7 @@
       <c r="B4" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="C4" s="150" t="s">
+      <c r="C4" s="117" t="s">
         <v>24</v>
       </c>
       <c r="D4" s="114"/>
@@ -2846,23 +2846,23 @@
         <v>4</v>
       </c>
       <c r="H4" s="114"/>
-      <c r="I4" s="153" t="s">
+      <c r="I4" s="120" t="s">
         <v>5</v>
       </c>
-      <c r="J4" s="154"/>
-      <c r="K4" s="151" t="s">
+      <c r="J4" s="121"/>
+      <c r="K4" s="118" t="s">
         <v>6</v>
       </c>
-      <c r="L4" s="152"/>
-      <c r="M4" s="151" t="s">
+      <c r="L4" s="119"/>
+      <c r="M4" s="118" t="s">
         <v>35</v>
       </c>
-      <c r="N4" s="152"/>
+      <c r="N4" s="119"/>
       <c r="O4" s="2"/>
     </row>
     <row r="5" spans="1:15" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2"/>
-      <c r="B5" s="137" t="s">
+      <c r="B5" s="136" t="s">
         <v>22</v>
       </c>
       <c r="C5" s="140" t="s">
@@ -2893,15 +2893,15 @@
       <c r="L5" s="41">
         <v>0.45833333333333331</v>
       </c>
-      <c r="M5" s="125"/>
-      <c r="N5" s="126"/>
+      <c r="M5" s="145"/>
+      <c r="N5" s="146"/>
       <c r="O5" s="2"/>
     </row>
     <row r="6" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A6" s="2"/>
-      <c r="B6" s="138"/>
-      <c r="C6" s="142"/>
-      <c r="D6" s="143"/>
+      <c r="B6" s="137"/>
+      <c r="C6" s="128"/>
+      <c r="D6" s="129"/>
       <c r="E6" s="45">
         <v>0.73958333333333337</v>
       </c>
@@ -2918,17 +2918,17 @@
       </c>
       <c r="K6" s="45"/>
       <c r="L6" s="46"/>
-      <c r="M6" s="117"/>
-      <c r="N6" s="118"/>
+      <c r="M6" s="147"/>
+      <c r="N6" s="148"/>
       <c r="O6" s="2"/>
     </row>
     <row r="7" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
-      <c r="B7" s="138"/>
-      <c r="C7" s="142" t="s">
+      <c r="B7" s="137"/>
+      <c r="C7" s="128" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="143"/>
+      <c r="D7" s="129"/>
       <c r="E7" s="40">
         <v>0.42708333333333331</v>
       </c>
@@ -2945,15 +2945,15 @@
       </c>
       <c r="K7" s="40"/>
       <c r="L7" s="41"/>
-      <c r="M7" s="125"/>
-      <c r="N7" s="126"/>
+      <c r="M7" s="145"/>
+      <c r="N7" s="146"/>
       <c r="O7" s="2"/>
     </row>
     <row r="8" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A8" s="2"/>
-      <c r="B8" s="138"/>
-      <c r="C8" s="142"/>
-      <c r="D8" s="143"/>
+      <c r="B8" s="137"/>
+      <c r="C8" s="128"/>
+      <c r="D8" s="129"/>
       <c r="E8" s="45">
         <v>0.77083333333333337</v>
       </c>
@@ -2970,17 +2970,17 @@
       </c>
       <c r="K8" s="47"/>
       <c r="L8" s="48"/>
-      <c r="M8" s="117"/>
-      <c r="N8" s="118"/>
+      <c r="M8" s="147"/>
+      <c r="N8" s="148"/>
       <c r="O8" s="10"/>
     </row>
     <row r="9" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A9" s="2"/>
-      <c r="B9" s="138"/>
-      <c r="C9" s="142" t="s">
+      <c r="B9" s="137"/>
+      <c r="C9" s="128" t="s">
         <v>27</v>
       </c>
-      <c r="D9" s="143"/>
+      <c r="D9" s="129"/>
       <c r="E9" s="40">
         <v>0.39583333333333331</v>
       </c>
@@ -3005,17 +3005,17 @@
       <c r="L9" s="41">
         <v>0.77083333333333337</v>
       </c>
-      <c r="M9" s="125"/>
-      <c r="N9" s="126"/>
+      <c r="M9" s="145"/>
+      <c r="N9" s="146"/>
       <c r="O9" s="10"/>
     </row>
     <row r="10" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A10" s="2"/>
-      <c r="B10" s="138"/>
-      <c r="C10" s="142" t="s">
+      <c r="B10" s="137"/>
+      <c r="C10" s="128" t="s">
         <v>28</v>
       </c>
-      <c r="D10" s="143"/>
+      <c r="D10" s="129"/>
       <c r="E10" s="45">
         <v>0.36458333333333331</v>
       </c>
@@ -3032,15 +3032,15 @@
       </c>
       <c r="K10" s="47"/>
       <c r="L10" s="48"/>
-      <c r="M10" s="117"/>
-      <c r="N10" s="118"/>
+      <c r="M10" s="147"/>
+      <c r="N10" s="148"/>
       <c r="O10" s="10"/>
     </row>
     <row r="11" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A11" s="2"/>
-      <c r="B11" s="138"/>
-      <c r="C11" s="142"/>
-      <c r="D11" s="143"/>
+      <c r="B11" s="137"/>
+      <c r="C11" s="128"/>
+      <c r="D11" s="129"/>
       <c r="E11" s="40">
         <v>0.66666666666666663</v>
       </c>
@@ -3057,17 +3057,17 @@
       </c>
       <c r="K11" s="40"/>
       <c r="L11" s="41"/>
-      <c r="M11" s="125"/>
-      <c r="N11" s="126"/>
+      <c r="M11" s="145"/>
+      <c r="N11" s="146"/>
       <c r="O11" s="10"/>
     </row>
     <row r="12" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>
-      <c r="B12" s="138"/>
-      <c r="C12" s="135" t="s">
+      <c r="B12" s="137"/>
+      <c r="C12" s="134" t="s">
         <v>29</v>
       </c>
-      <c r="D12" s="136"/>
+      <c r="D12" s="135"/>
       <c r="E12" s="45">
         <v>0.33333333333333331</v>
       </c>
@@ -3084,17 +3084,17 @@
       </c>
       <c r="K12" s="45"/>
       <c r="L12" s="46"/>
-      <c r="M12" s="117" t="s">
+      <c r="M12" s="147" t="s">
         <v>36</v>
       </c>
-      <c r="N12" s="118"/>
+      <c r="N12" s="148"/>
       <c r="O12" s="10"/>
     </row>
     <row r="13" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A13" s="2"/>
-      <c r="B13" s="138"/>
-      <c r="C13" s="135"/>
-      <c r="D13" s="136"/>
+      <c r="B13" s="137"/>
+      <c r="C13" s="134"/>
+      <c r="D13" s="135"/>
       <c r="E13" s="40">
         <v>0.45833333333333331</v>
       </c>
@@ -3111,15 +3111,15 @@
       </c>
       <c r="K13" s="40"/>
       <c r="L13" s="41"/>
-      <c r="M13" s="125"/>
-      <c r="N13" s="126"/>
+      <c r="M13" s="145"/>
+      <c r="N13" s="146"/>
       <c r="O13" s="10"/>
     </row>
     <row r="14" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A14" s="2"/>
-      <c r="B14" s="138"/>
-      <c r="C14" s="135"/>
-      <c r="D14" s="136"/>
+      <c r="B14" s="137"/>
+      <c r="C14" s="134"/>
+      <c r="D14" s="135"/>
       <c r="E14" s="45"/>
       <c r="F14" s="46"/>
       <c r="G14" s="45">
@@ -3136,15 +3136,15 @@
       <c r="L14" s="46">
         <v>0.72916666666666663</v>
       </c>
-      <c r="M14" s="117"/>
-      <c r="N14" s="118"/>
+      <c r="M14" s="147"/>
+      <c r="N14" s="148"/>
       <c r="O14" s="10"/>
     </row>
     <row r="15" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A15" s="2"/>
-      <c r="B15" s="138"/>
-      <c r="C15" s="135"/>
-      <c r="D15" s="136"/>
+      <c r="B15" s="137"/>
+      <c r="C15" s="134"/>
+      <c r="D15" s="135"/>
       <c r="E15" s="40"/>
       <c r="F15" s="41"/>
       <c r="G15" s="40">
@@ -3161,19 +3161,19 @@
       <c r="L15" s="41">
         <v>0.77083333333333337</v>
       </c>
-      <c r="M15" s="125"/>
-      <c r="N15" s="126"/>
+      <c r="M15" s="145"/>
+      <c r="N15" s="146"/>
       <c r="O15" s="10"/>
     </row>
     <row r="16" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
-      <c r="B16" s="139" t="s">
+      <c r="B16" s="130" t="s">
         <v>31</v>
       </c>
-      <c r="C16" s="144" t="s">
+      <c r="C16" s="124" t="s">
         <v>27</v>
       </c>
-      <c r="D16" s="133"/>
+      <c r="D16" s="125"/>
       <c r="E16" s="8"/>
       <c r="F16" s="9"/>
       <c r="G16" s="8">
@@ -3190,15 +3190,15 @@
       <c r="L16" s="9">
         <v>0.42708333333333331</v>
       </c>
-      <c r="M16" s="123"/>
-      <c r="N16" s="124"/>
+      <c r="M16" s="153"/>
+      <c r="N16" s="154"/>
       <c r="O16" s="10"/>
     </row>
     <row r="17" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A17" s="2"/>
-      <c r="B17" s="139"/>
-      <c r="C17" s="144"/>
-      <c r="D17" s="133"/>
+      <c r="B17" s="130"/>
+      <c r="C17" s="124"/>
+      <c r="D17" s="125"/>
       <c r="E17" s="8"/>
       <c r="F17" s="9"/>
       <c r="G17" s="8">
@@ -3215,17 +3215,17 @@
       <c r="L17" s="9">
         <v>0.80208333333333337</v>
       </c>
-      <c r="M17" s="123"/>
-      <c r="N17" s="124"/>
+      <c r="M17" s="153"/>
+      <c r="N17" s="154"/>
       <c r="O17" s="10"/>
     </row>
     <row r="18" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A18" s="2"/>
-      <c r="B18" s="139"/>
-      <c r="C18" s="144" t="s">
+      <c r="B18" s="130"/>
+      <c r="C18" s="124" t="s">
         <v>28</v>
       </c>
-      <c r="D18" s="133"/>
+      <c r="D18" s="125"/>
       <c r="E18" s="8"/>
       <c r="F18" s="9"/>
       <c r="G18" s="8">
@@ -3242,15 +3242,15 @@
       <c r="L18" s="9">
         <v>0.39583333333333331</v>
       </c>
-      <c r="M18" s="123"/>
-      <c r="N18" s="124"/>
+      <c r="M18" s="153"/>
+      <c r="N18" s="154"/>
       <c r="O18" s="10"/>
     </row>
     <row r="19" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A19" s="2"/>
-      <c r="B19" s="139"/>
-      <c r="C19" s="144"/>
-      <c r="D19" s="133"/>
+      <c r="B19" s="130"/>
+      <c r="C19" s="124"/>
+      <c r="D19" s="125"/>
       <c r="E19" s="8"/>
       <c r="F19" s="9"/>
       <c r="G19" s="8">
@@ -3267,17 +3267,17 @@
       <c r="L19" s="9">
         <v>0.69791666666666663</v>
       </c>
-      <c r="M19" s="123"/>
-      <c r="N19" s="124"/>
+      <c r="M19" s="153"/>
+      <c r="N19" s="154"/>
       <c r="O19" s="10"/>
     </row>
     <row r="20" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A20" s="2"/>
-      <c r="B20" s="139"/>
-      <c r="C20" s="145" t="s">
+      <c r="B20" s="130"/>
+      <c r="C20" s="126" t="s">
         <v>29</v>
       </c>
-      <c r="D20" s="146"/>
+      <c r="D20" s="127"/>
       <c r="E20" s="8"/>
       <c r="F20" s="9"/>
       <c r="G20" s="8">
@@ -3294,17 +3294,17 @@
       <c r="L20" s="9">
         <v>0.36458333333333331</v>
       </c>
-      <c r="M20" s="123" t="s">
+      <c r="M20" s="153" t="s">
         <v>37</v>
       </c>
-      <c r="N20" s="124"/>
+      <c r="N20" s="154"/>
       <c r="O20" s="10"/>
     </row>
     <row r="21" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A21" s="2"/>
-      <c r="B21" s="139"/>
-      <c r="C21" s="145"/>
-      <c r="D21" s="146"/>
+      <c r="B21" s="130"/>
+      <c r="C21" s="126"/>
+      <c r="D21" s="127"/>
       <c r="E21" s="8"/>
       <c r="F21" s="9"/>
       <c r="G21" s="8">
@@ -3321,19 +3321,19 @@
       <c r="L21" s="9">
         <v>0.83333333333333337</v>
       </c>
-      <c r="M21" s="123"/>
-      <c r="N21" s="124"/>
+      <c r="M21" s="153"/>
+      <c r="N21" s="154"/>
       <c r="O21" s="10"/>
     </row>
     <row r="22" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A22" s="2"/>
-      <c r="B22" s="138" t="s">
+      <c r="B22" s="137" t="s">
         <v>33</v>
       </c>
-      <c r="C22" s="142" t="s">
+      <c r="C22" s="128" t="s">
         <v>28</v>
       </c>
-      <c r="D22" s="143"/>
+      <c r="D22" s="129"/>
       <c r="E22" s="45">
         <v>0.69791666666666663</v>
       </c>
@@ -3350,17 +3350,17 @@
       </c>
       <c r="K22" s="45"/>
       <c r="L22" s="46"/>
-      <c r="M22" s="117"/>
-      <c r="N22" s="118"/>
+      <c r="M22" s="147"/>
+      <c r="N22" s="148"/>
       <c r="O22" s="10"/>
     </row>
     <row r="23" spans="1:15" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2"/>
-      <c r="B23" s="138"/>
-      <c r="C23" s="142" t="s">
+      <c r="B23" s="137"/>
+      <c r="C23" s="128" t="s">
         <v>29</v>
       </c>
-      <c r="D23" s="143"/>
+      <c r="D23" s="129"/>
       <c r="E23" s="45">
         <v>0.80208333333333337</v>
       </c>
@@ -3377,52 +3377,52 @@
       </c>
       <c r="K23" s="45"/>
       <c r="L23" s="46"/>
-      <c r="M23" s="117"/>
-      <c r="N23" s="118"/>
+      <c r="M23" s="147"/>
+      <c r="N23" s="148"/>
       <c r="O23" s="10"/>
     </row>
     <row r="24" spans="1:15" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2"/>
-      <c r="B24" s="139" t="s">
+      <c r="B24" s="130" t="s">
         <v>30</v>
       </c>
-      <c r="C24" s="145"/>
-      <c r="D24" s="146"/>
-      <c r="E24" s="127">
+      <c r="C24" s="126"/>
+      <c r="D24" s="127"/>
+      <c r="E24" s="138">
         <v>0.5</v>
       </c>
-      <c r="F24" s="129">
+      <c r="F24" s="122">
         <v>0.53125</v>
       </c>
-      <c r="G24" s="127"/>
-      <c r="H24" s="129"/>
-      <c r="I24" s="131">
+      <c r="G24" s="138"/>
+      <c r="H24" s="122"/>
+      <c r="I24" s="142">
         <v>0.5</v>
       </c>
-      <c r="J24" s="133">
+      <c r="J24" s="125">
         <v>0.53125</v>
       </c>
-      <c r="K24" s="127"/>
-      <c r="L24" s="133"/>
-      <c r="M24" s="119"/>
-      <c r="N24" s="120"/>
+      <c r="K24" s="138"/>
+      <c r="L24" s="125"/>
+      <c r="M24" s="149"/>
+      <c r="N24" s="150"/>
       <c r="O24" s="10"/>
     </row>
     <row r="25" spans="1:15" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="2"/>
-      <c r="B25" s="147"/>
-      <c r="C25" s="148"/>
-      <c r="D25" s="149"/>
-      <c r="E25" s="128"/>
-      <c r="F25" s="130"/>
-      <c r="G25" s="128"/>
-      <c r="H25" s="130"/>
-      <c r="I25" s="132"/>
-      <c r="J25" s="134"/>
-      <c r="K25" s="128"/>
-      <c r="L25" s="134"/>
-      <c r="M25" s="121"/>
-      <c r="N25" s="122"/>
+      <c r="B25" s="131"/>
+      <c r="C25" s="132"/>
+      <c r="D25" s="133"/>
+      <c r="E25" s="139"/>
+      <c r="F25" s="123"/>
+      <c r="G25" s="139"/>
+      <c r="H25" s="123"/>
+      <c r="I25" s="143"/>
+      <c r="J25" s="144"/>
+      <c r="K25" s="139"/>
+      <c r="L25" s="144"/>
+      <c r="M25" s="151"/>
+      <c r="N25" s="152"/>
       <c r="O25" s="10"/>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
@@ -3463,35 +3463,15 @@
     </row>
   </sheetData>
   <mergeCells count="49">
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="E4:F4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="M4:N4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="K4:L4"/>
-    <mergeCell ref="F24:F25"/>
-    <mergeCell ref="C16:D17"/>
-    <mergeCell ref="C18:D19"/>
-    <mergeCell ref="C20:D21"/>
-    <mergeCell ref="C22:D22"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="B24:D25"/>
-    <mergeCell ref="C12:D15"/>
-    <mergeCell ref="B5:B15"/>
-    <mergeCell ref="B16:B21"/>
-    <mergeCell ref="B22:B23"/>
-    <mergeCell ref="E24:E25"/>
-    <mergeCell ref="C5:D6"/>
-    <mergeCell ref="C7:D8"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="C10:D11"/>
-    <mergeCell ref="G24:G25"/>
-    <mergeCell ref="H24:H25"/>
-    <mergeCell ref="I24:I25"/>
-    <mergeCell ref="L24:L25"/>
-    <mergeCell ref="J24:J25"/>
-    <mergeCell ref="K24:K25"/>
+    <mergeCell ref="M22:N22"/>
+    <mergeCell ref="M23:N23"/>
+    <mergeCell ref="M24:N25"/>
+    <mergeCell ref="M16:N16"/>
+    <mergeCell ref="M17:N17"/>
+    <mergeCell ref="M18:N18"/>
+    <mergeCell ref="M19:N19"/>
+    <mergeCell ref="M20:N20"/>
+    <mergeCell ref="M21:N21"/>
     <mergeCell ref="M15:N15"/>
     <mergeCell ref="M5:N5"/>
     <mergeCell ref="M6:N6"/>
@@ -3503,15 +3483,35 @@
     <mergeCell ref="M12:N12"/>
     <mergeCell ref="M13:N13"/>
     <mergeCell ref="M14:N14"/>
-    <mergeCell ref="M22:N22"/>
-    <mergeCell ref="M23:N23"/>
-    <mergeCell ref="M24:N25"/>
-    <mergeCell ref="M16:N16"/>
-    <mergeCell ref="M17:N17"/>
-    <mergeCell ref="M18:N18"/>
-    <mergeCell ref="M19:N19"/>
-    <mergeCell ref="M20:N20"/>
-    <mergeCell ref="M21:N21"/>
+    <mergeCell ref="G24:G25"/>
+    <mergeCell ref="H24:H25"/>
+    <mergeCell ref="I24:I25"/>
+    <mergeCell ref="L24:L25"/>
+    <mergeCell ref="J24:J25"/>
+    <mergeCell ref="K24:K25"/>
+    <mergeCell ref="C12:D15"/>
+    <mergeCell ref="B5:B15"/>
+    <mergeCell ref="B16:B21"/>
+    <mergeCell ref="B22:B23"/>
+    <mergeCell ref="E24:E25"/>
+    <mergeCell ref="C5:D6"/>
+    <mergeCell ref="C7:D8"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="C10:D11"/>
+    <mergeCell ref="F24:F25"/>
+    <mergeCell ref="C16:D17"/>
+    <mergeCell ref="C18:D19"/>
+    <mergeCell ref="C20:D21"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="B24:D25"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="K4:L4"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
@@ -3584,23 +3584,23 @@
       <c r="D3" s="157" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="152"/>
-      <c r="F3" s="151" t="s">
+      <c r="E3" s="119"/>
+      <c r="F3" s="118" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="152"/>
-      <c r="H3" s="151" t="s">
+      <c r="G3" s="119"/>
+      <c r="H3" s="118" t="s">
         <v>4</v>
       </c>
-      <c r="I3" s="152"/>
-      <c r="J3" s="151" t="s">
+      <c r="I3" s="119"/>
+      <c r="J3" s="118" t="s">
         <v>5</v>
       </c>
-      <c r="K3" s="152"/>
-      <c r="L3" s="151" t="s">
+      <c r="K3" s="119"/>
+      <c r="L3" s="118" t="s">
         <v>6</v>
       </c>
-      <c r="M3" s="152"/>
+      <c r="M3" s="119"/>
       <c r="N3" s="2"/>
     </row>
     <row r="4" spans="1:14" ht="18.75" x14ac:dyDescent="0.25">
@@ -4115,10 +4115,10 @@
       <c r="E4" s="65" t="s">
         <v>68</v>
       </c>
-      <c r="F4" s="179" t="s">
+      <c r="F4" s="170" t="s">
         <v>69</v>
       </c>
-      <c r="G4" s="179"/>
+      <c r="G4" s="170"/>
       <c r="H4" s="66" t="s">
         <v>73</v>
       </c>
@@ -4129,10 +4129,10 @@
     </row>
     <row r="5" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A5" s="2"/>
-      <c r="B5" s="164" t="s">
+      <c r="B5" s="189" t="s">
         <v>66</v>
       </c>
-      <c r="C5" s="131" t="s">
+      <c r="C5" s="142" t="s">
         <v>40</v>
       </c>
       <c r="D5" s="16" t="s">
@@ -4147,18 +4147,18 @@
       <c r="G5" s="16">
         <v>0.39583333333333331</v>
       </c>
-      <c r="H5" s="187">
+      <c r="H5" s="178">
         <v>10</v>
       </c>
-      <c r="I5" s="133" t="s">
+      <c r="I5" s="125" t="s">
         <v>90</v>
       </c>
       <c r="J5" s="2"/>
     </row>
     <row r="6" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2"/>
-      <c r="B6" s="164"/>
-      <c r="C6" s="132"/>
+      <c r="B6" s="189"/>
+      <c r="C6" s="143"/>
       <c r="D6" s="67" t="s">
         <v>46</v>
       </c>
@@ -4171,14 +4171,14 @@
       <c r="G6" s="67">
         <v>0.75</v>
       </c>
-      <c r="H6" s="188"/>
-      <c r="I6" s="134"/>
+      <c r="H6" s="179"/>
+      <c r="I6" s="144"/>
       <c r="J6" s="2"/>
     </row>
     <row r="7" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
-      <c r="B7" s="164"/>
-      <c r="C7" s="166" t="s">
+      <c r="B7" s="189"/>
+      <c r="C7" s="191" t="s">
         <v>43</v>
       </c>
       <c r="D7" s="72" t="s">
@@ -4193,18 +4193,18 @@
       <c r="G7" s="69">
         <v>0.41666666666666669</v>
       </c>
-      <c r="H7" s="183">
+      <c r="H7" s="174">
         <v>16</v>
       </c>
-      <c r="I7" s="180" t="s">
+      <c r="I7" s="171" t="s">
         <v>91</v>
       </c>
       <c r="J7" s="2"/>
     </row>
     <row r="8" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A8" s="2"/>
-      <c r="B8" s="164"/>
-      <c r="C8" s="167"/>
+      <c r="B8" s="189"/>
+      <c r="C8" s="192"/>
       <c r="D8" s="23" t="s">
         <v>48</v>
       </c>
@@ -4217,14 +4217,14 @@
       <c r="G8" s="60">
         <v>0.76041666666666663</v>
       </c>
-      <c r="H8" s="184"/>
-      <c r="I8" s="176"/>
+      <c r="H8" s="175"/>
+      <c r="I8" s="167"/>
       <c r="J8" s="10"/>
     </row>
     <row r="9" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A9" s="2"/>
-      <c r="B9" s="164"/>
-      <c r="C9" s="167"/>
+      <c r="B9" s="189"/>
+      <c r="C9" s="192"/>
       <c r="D9" s="23" t="s">
         <v>49</v>
       </c>
@@ -4237,28 +4237,28 @@
       <c r="G9" s="60">
         <v>0.79166666666666663</v>
       </c>
-      <c r="H9" s="184"/>
-      <c r="I9" s="176" t="s">
+      <c r="H9" s="175"/>
+      <c r="I9" s="167" t="s">
         <v>92</v>
       </c>
       <c r="J9" s="10"/>
     </row>
     <row r="10" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2"/>
-      <c r="B10" s="164"/>
-      <c r="C10" s="168"/>
+      <c r="B10" s="189"/>
+      <c r="C10" s="193"/>
       <c r="D10" s="30"/>
       <c r="E10" s="71"/>
       <c r="F10" s="71"/>
       <c r="G10" s="71"/>
-      <c r="H10" s="185"/>
-      <c r="I10" s="177"/>
+      <c r="H10" s="176"/>
+      <c r="I10" s="168"/>
       <c r="J10" s="10"/>
     </row>
     <row r="11" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A11" s="2"/>
-      <c r="B11" s="164"/>
-      <c r="C11" s="169" t="s">
+      <c r="B11" s="189"/>
+      <c r="C11" s="194" t="s">
         <v>71</v>
       </c>
       <c r="D11" s="75" t="s">
@@ -4273,7 +4273,7 @@
       <c r="G11" s="76">
         <v>0.45833333333333331</v>
       </c>
-      <c r="H11" s="189">
+      <c r="H11" s="180">
         <v>14</v>
       </c>
       <c r="I11" s="77" t="s">
@@ -4283,8 +4283,8 @@
     </row>
     <row r="12" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>
-      <c r="B12" s="164"/>
-      <c r="C12" s="170"/>
+      <c r="B12" s="189"/>
+      <c r="C12" s="195"/>
       <c r="D12" s="78" t="s">
         <v>74</v>
       </c>
@@ -4297,7 +4297,7 @@
       <c r="G12" s="61">
         <v>0.45833333333333331</v>
       </c>
-      <c r="H12" s="190"/>
+      <c r="H12" s="181"/>
       <c r="I12" s="57" t="s">
         <v>91</v>
       </c>
@@ -4305,8 +4305,8 @@
     </row>
     <row r="13" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A13" s="2"/>
-      <c r="B13" s="164"/>
-      <c r="C13" s="170"/>
+      <c r="B13" s="189"/>
+      <c r="C13" s="195"/>
       <c r="D13" s="78" t="s">
         <v>74</v>
       </c>
@@ -4319,16 +4319,16 @@
       <c r="G13" s="61">
         <v>0.77083333333333337</v>
       </c>
-      <c r="H13" s="190"/>
-      <c r="I13" s="181" t="s">
+      <c r="H13" s="181"/>
+      <c r="I13" s="172" t="s">
         <v>93</v>
       </c>
       <c r="J13" s="10"/>
     </row>
     <row r="14" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A14" s="2"/>
-      <c r="B14" s="164"/>
-      <c r="C14" s="170"/>
+      <c r="B14" s="189"/>
+      <c r="C14" s="195"/>
       <c r="D14" s="78" t="s">
         <v>75</v>
       </c>
@@ -4341,14 +4341,14 @@
       <c r="G14" s="61">
         <v>0.45833333333333331</v>
       </c>
-      <c r="H14" s="190"/>
-      <c r="I14" s="181"/>
+      <c r="H14" s="181"/>
+      <c r="I14" s="172"/>
       <c r="J14" s="10"/>
     </row>
     <row r="15" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A15" s="2"/>
-      <c r="B15" s="164"/>
-      <c r="C15" s="170"/>
+      <c r="B15" s="189"/>
+      <c r="C15" s="195"/>
       <c r="D15" s="78" t="s">
         <v>75</v>
       </c>
@@ -4361,14 +4361,14 @@
       <c r="G15" s="61">
         <v>0.80208333333333337</v>
       </c>
-      <c r="H15" s="190"/>
-      <c r="I15" s="181"/>
+      <c r="H15" s="181"/>
+      <c r="I15" s="172"/>
       <c r="J15" s="10"/>
     </row>
     <row r="16" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
-      <c r="B16" s="164"/>
-      <c r="C16" s="170"/>
+      <c r="B16" s="189"/>
+      <c r="C16" s="195"/>
       <c r="D16" s="78" t="s">
         <v>76</v>
       </c>
@@ -4381,14 +4381,14 @@
       <c r="G16" s="61">
         <v>0.42708333333333331</v>
       </c>
-      <c r="H16" s="190"/>
-      <c r="I16" s="181"/>
+      <c r="H16" s="181"/>
+      <c r="I16" s="172"/>
       <c r="J16" s="10"/>
     </row>
     <row r="17" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A17" s="2"/>
-      <c r="B17" s="164"/>
-      <c r="C17" s="170"/>
+      <c r="B17" s="189"/>
+      <c r="C17" s="195"/>
       <c r="D17" s="78" t="s">
         <v>76</v>
       </c>
@@ -4401,14 +4401,14 @@
       <c r="G17" s="61">
         <v>0.77083333333333337</v>
       </c>
-      <c r="H17" s="190"/>
-      <c r="I17" s="181"/>
+      <c r="H17" s="181"/>
+      <c r="I17" s="172"/>
       <c r="J17" s="10"/>
     </row>
     <row r="18" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A18" s="2"/>
-      <c r="B18" s="164"/>
-      <c r="C18" s="170"/>
+      <c r="B18" s="189"/>
+      <c r="C18" s="195"/>
       <c r="D18" s="78" t="s">
         <v>77</v>
       </c>
@@ -4421,14 +4421,14 @@
       <c r="G18" s="61">
         <v>0.39583333333333331</v>
       </c>
-      <c r="H18" s="190"/>
-      <c r="I18" s="181"/>
+      <c r="H18" s="181"/>
+      <c r="I18" s="172"/>
       <c r="J18" s="10"/>
     </row>
     <row r="19" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2"/>
-      <c r="B19" s="164"/>
-      <c r="C19" s="170"/>
+      <c r="B19" s="189"/>
+      <c r="C19" s="195"/>
       <c r="D19" s="79" t="s">
         <v>77</v>
       </c>
@@ -4441,14 +4441,14 @@
       <c r="G19" s="80">
         <v>0.69791666666666663</v>
       </c>
-      <c r="H19" s="191"/>
-      <c r="I19" s="182"/>
+      <c r="H19" s="182"/>
+      <c r="I19" s="173"/>
       <c r="J19" s="10"/>
     </row>
     <row r="20" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A20" s="2"/>
-      <c r="B20" s="164"/>
-      <c r="C20" s="170"/>
+      <c r="B20" s="189"/>
+      <c r="C20" s="195"/>
       <c r="D20" s="81" t="s">
         <v>78</v>
       </c>
@@ -4461,7 +4461,7 @@
       <c r="G20" s="82">
         <v>0.36458333333333331</v>
       </c>
-      <c r="H20" s="192">
+      <c r="H20" s="183">
         <v>12</v>
       </c>
       <c r="I20" s="83" t="s">
@@ -4471,8 +4471,8 @@
     </row>
     <row r="21" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A21" s="2"/>
-      <c r="B21" s="164"/>
-      <c r="C21" s="170"/>
+      <c r="B21" s="189"/>
+      <c r="C21" s="195"/>
       <c r="D21" s="84" t="s">
         <v>78</v>
       </c>
@@ -4485,7 +4485,7 @@
       <c r="G21" s="62">
         <v>0.48958333333333331</v>
       </c>
-      <c r="H21" s="193"/>
+      <c r="H21" s="184"/>
       <c r="I21" s="58" t="s">
         <v>94</v>
       </c>
@@ -4493,8 +4493,8 @@
     </row>
     <row r="22" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A22" s="2"/>
-      <c r="B22" s="164"/>
-      <c r="C22" s="170"/>
+      <c r="B22" s="189"/>
+      <c r="C22" s="195"/>
       <c r="D22" s="84" t="s">
         <v>78</v>
       </c>
@@ -4507,7 +4507,7 @@
       <c r="G22" s="62">
         <v>0.72916666666666663</v>
       </c>
-      <c r="H22" s="193"/>
+      <c r="H22" s="184"/>
       <c r="I22" s="58" t="s">
         <v>93</v>
       </c>
@@ -4515,8 +4515,8 @@
     </row>
     <row r="23" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A23" s="2"/>
-      <c r="B23" s="164"/>
-      <c r="C23" s="170"/>
+      <c r="B23" s="189"/>
+      <c r="C23" s="195"/>
       <c r="D23" s="84" t="s">
         <v>78</v>
       </c>
@@ -4529,7 +4529,7 @@
       <c r="G23" s="62">
         <v>0.77083333333333337</v>
       </c>
-      <c r="H23" s="193"/>
+      <c r="H23" s="184"/>
       <c r="I23" s="58" t="s">
         <v>92</v>
       </c>
@@ -4537,8 +4537,8 @@
     </row>
     <row r="24" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="2"/>
-      <c r="B24" s="164"/>
-      <c r="C24" s="170"/>
+      <c r="B24" s="189"/>
+      <c r="C24" s="195"/>
       <c r="D24" s="85" t="s">
         <v>78</v>
       </c>
@@ -4551,7 +4551,7 @@
       <c r="G24" s="86">
         <v>0.46875</v>
       </c>
-      <c r="H24" s="194"/>
+      <c r="H24" s="185"/>
       <c r="I24" s="87" t="s">
         <v>94</v>
       </c>
@@ -4559,8 +4559,8 @@
     </row>
     <row r="25" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A25" s="2"/>
-      <c r="B25" s="164"/>
-      <c r="C25" s="170"/>
+      <c r="B25" s="189"/>
+      <c r="C25" s="195"/>
       <c r="D25" s="88" t="s">
         <v>79</v>
       </c>
@@ -4573,18 +4573,18 @@
       <c r="G25" s="89">
         <v>0.42708333333333331</v>
       </c>
-      <c r="H25" s="195">
+      <c r="H25" s="186">
         <v>14</v>
       </c>
-      <c r="I25" s="173" t="s">
+      <c r="I25" s="164" t="s">
         <v>93</v>
       </c>
       <c r="J25" s="10"/>
     </row>
     <row r="26" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A26" s="2"/>
-      <c r="B26" s="164"/>
-      <c r="C26" s="170"/>
+      <c r="B26" s="189"/>
+      <c r="C26" s="195"/>
       <c r="D26" s="90" t="s">
         <v>79</v>
       </c>
@@ -4597,14 +4597,14 @@
       <c r="G26" s="63">
         <v>0.80208333333333337</v>
       </c>
-      <c r="H26" s="196"/>
-      <c r="I26" s="174"/>
+      <c r="H26" s="187"/>
+      <c r="I26" s="165"/>
       <c r="J26" s="10"/>
     </row>
     <row r="27" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A27" s="2"/>
-      <c r="B27" s="164"/>
-      <c r="C27" s="170"/>
+      <c r="B27" s="189"/>
+      <c r="C27" s="195"/>
       <c r="D27" s="90" t="s">
         <v>80</v>
       </c>
@@ -4617,14 +4617,14 @@
       <c r="G27" s="63">
         <v>0.39583333333333331</v>
       </c>
-      <c r="H27" s="196"/>
-      <c r="I27" s="174"/>
+      <c r="H27" s="187"/>
+      <c r="I27" s="165"/>
       <c r="J27" s="10"/>
     </row>
     <row r="28" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="2"/>
-      <c r="B28" s="164"/>
-      <c r="C28" s="170"/>
+      <c r="B28" s="189"/>
+      <c r="C28" s="195"/>
       <c r="D28" s="91" t="s">
         <v>80</v>
       </c>
@@ -4637,14 +4637,14 @@
       <c r="G28" s="92">
         <v>0.69791666666666663</v>
       </c>
-      <c r="H28" s="197"/>
-      <c r="I28" s="175"/>
+      <c r="H28" s="188"/>
+      <c r="I28" s="166"/>
       <c r="J28" s="10"/>
     </row>
     <row r="29" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A29" s="2"/>
-      <c r="B29" s="164"/>
-      <c r="C29" s="170"/>
+      <c r="B29" s="189"/>
+      <c r="C29" s="195"/>
       <c r="D29" s="93" t="s">
         <v>81</v>
       </c>
@@ -4657,7 +4657,7 @@
       <c r="G29" s="69">
         <v>0.36458333333333331</v>
       </c>
-      <c r="H29" s="183">
+      <c r="H29" s="174">
         <v>12</v>
       </c>
       <c r="I29" s="94" t="s">
@@ -4667,8 +4667,8 @@
     </row>
     <row r="30" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A30" s="2"/>
-      <c r="B30" s="164"/>
-      <c r="C30" s="170"/>
+      <c r="B30" s="189"/>
+      <c r="C30" s="195"/>
       <c r="D30" s="25" t="s">
         <v>81</v>
       </c>
@@ -4681,16 +4681,16 @@
       <c r="G30" s="60">
         <v>0.83333333333333337</v>
       </c>
-      <c r="H30" s="184"/>
-      <c r="I30" s="176" t="s">
+      <c r="H30" s="175"/>
+      <c r="I30" s="167" t="s">
         <v>94</v>
       </c>
       <c r="J30" s="10"/>
     </row>
     <row r="31" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="2"/>
-      <c r="B31" s="164"/>
-      <c r="C31" s="170"/>
+      <c r="B31" s="189"/>
+      <c r="C31" s="195"/>
       <c r="D31" s="33" t="s">
         <v>81</v>
       </c>
@@ -4703,14 +4703,14 @@
       <c r="G31" s="70">
         <v>0.41666666666666669</v>
       </c>
-      <c r="H31" s="185"/>
-      <c r="I31" s="177"/>
+      <c r="H31" s="176"/>
+      <c r="I31" s="168"/>
       <c r="J31" s="10"/>
     </row>
     <row r="32" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A32" s="2"/>
-      <c r="B32" s="164"/>
-      <c r="C32" s="170"/>
+      <c r="B32" s="189"/>
+      <c r="C32" s="195"/>
       <c r="D32" s="75" t="s">
         <v>83</v>
       </c>
@@ -4733,8 +4733,8 @@
     </row>
     <row r="33" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A33" s="2"/>
-      <c r="B33" s="164"/>
-      <c r="C33" s="170"/>
+      <c r="B33" s="189"/>
+      <c r="C33" s="195"/>
       <c r="D33" s="84" t="s">
         <v>84</v>
       </c>
@@ -4757,8 +4757,8 @@
     </row>
     <row r="34" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="2"/>
-      <c r="B34" s="164"/>
-      <c r="C34" s="171"/>
+      <c r="B34" s="189"/>
+      <c r="C34" s="196"/>
       <c r="D34" s="79" t="s">
         <v>82</v>
       </c>
@@ -4781,8 +4781,8 @@
     </row>
     <row r="35" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A35" s="2"/>
-      <c r="B35" s="164"/>
-      <c r="C35" s="172" t="s">
+      <c r="B35" s="189"/>
+      <c r="C35" s="197" t="s">
         <v>44</v>
       </c>
       <c r="D35" s="99" t="s">
@@ -4797,7 +4797,7 @@
       <c r="G35" s="69">
         <v>0.77083333333333337</v>
       </c>
-      <c r="H35" s="183">
+      <c r="H35" s="174">
         <v>20</v>
       </c>
       <c r="I35" s="100" t="s">
@@ -4807,7 +4807,7 @@
     </row>
     <row r="36" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A36" s="2"/>
-      <c r="B36" s="164"/>
+      <c r="B36" s="189"/>
       <c r="C36" s="155"/>
       <c r="D36" s="27" t="s">
         <v>48</v>
@@ -4821,7 +4821,7 @@
       <c r="G36" s="60">
         <v>0.78472222222222221</v>
       </c>
-      <c r="H36" s="184"/>
+      <c r="H36" s="175"/>
       <c r="I36" s="24" t="s">
         <v>94</v>
       </c>
@@ -4829,7 +4829,7 @@
     </row>
     <row r="37" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A37" s="2"/>
-      <c r="B37" s="164"/>
+      <c r="B37" s="189"/>
       <c r="C37" s="155"/>
       <c r="D37" s="27" t="s">
         <v>49</v>
@@ -4843,7 +4843,7 @@
       <c r="G37" s="60">
         <v>0.80555555555555558</v>
       </c>
-      <c r="H37" s="184"/>
+      <c r="H37" s="175"/>
       <c r="I37" s="24" t="s">
         <v>91</v>
       </c>
@@ -4851,7 +4851,7 @@
     </row>
     <row r="38" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A38" s="2"/>
-      <c r="B38" s="164"/>
+      <c r="B38" s="189"/>
       <c r="C38" s="155"/>
       <c r="D38" s="27" t="s">
         <v>49</v>
@@ -4865,7 +4865,7 @@
       <c r="G38" s="60">
         <v>0.81944444444444442</v>
       </c>
-      <c r="H38" s="184"/>
+      <c r="H38" s="175"/>
       <c r="I38" s="24" t="s">
         <v>94</v>
       </c>
@@ -4873,7 +4873,7 @@
     </row>
     <row r="39" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A39" s="2"/>
-      <c r="B39" s="164"/>
+      <c r="B39" s="189"/>
       <c r="C39" s="155"/>
       <c r="D39" s="27" t="s">
         <v>50</v>
@@ -4887,7 +4887,7 @@
       <c r="G39" s="60">
         <v>0.84027777777777779</v>
       </c>
-      <c r="H39" s="184"/>
+      <c r="H39" s="175"/>
       <c r="I39" s="24" t="s">
         <v>91</v>
       </c>
@@ -4895,7 +4895,7 @@
     </row>
     <row r="40" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A40" s="2"/>
-      <c r="B40" s="164"/>
+      <c r="B40" s="189"/>
       <c r="C40" s="155"/>
       <c r="D40" s="27" t="s">
         <v>50</v>
@@ -4909,7 +4909,7 @@
       <c r="G40" s="60">
         <v>0.85416666666666663</v>
       </c>
-      <c r="H40" s="184"/>
+      <c r="H40" s="175"/>
       <c r="I40" s="24" t="s">
         <v>94</v>
       </c>
@@ -4917,7 +4917,7 @@
     </row>
     <row r="41" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="2"/>
-      <c r="B41" s="164"/>
+      <c r="B41" s="189"/>
       <c r="C41" s="156"/>
       <c r="D41" s="32" t="s">
         <v>51</v>
@@ -4931,7 +4931,7 @@
       <c r="G41" s="70">
         <v>0.72222222222222221</v>
       </c>
-      <c r="H41" s="185"/>
+      <c r="H41" s="176"/>
       <c r="I41" s="31" t="s">
         <v>91</v>
       </c>
@@ -4939,8 +4939,8 @@
     </row>
     <row r="42" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A42" s="2"/>
-      <c r="B42" s="164"/>
-      <c r="C42" s="169" t="s">
+      <c r="B42" s="189"/>
+      <c r="C42" s="194" t="s">
         <v>72</v>
       </c>
       <c r="D42" s="101" t="s">
@@ -4955,18 +4955,18 @@
       <c r="G42" s="102">
         <v>0.44444444444444442</v>
       </c>
-      <c r="H42" s="186">
+      <c r="H42" s="177">
         <v>12</v>
       </c>
-      <c r="I42" s="178" t="s">
+      <c r="I42" s="169" t="s">
         <v>94</v>
       </c>
       <c r="J42" s="10"/>
     </row>
     <row r="43" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A43" s="2"/>
-      <c r="B43" s="164"/>
-      <c r="C43" s="170"/>
+      <c r="B43" s="189"/>
+      <c r="C43" s="195"/>
       <c r="D43" s="15" t="s">
         <v>48</v>
       </c>
@@ -4979,14 +4979,14 @@
       <c r="G43" s="16">
         <v>0.44444444444444442</v>
       </c>
-      <c r="H43" s="187"/>
-      <c r="I43" s="133"/>
+      <c r="H43" s="178"/>
+      <c r="I43" s="125"/>
       <c r="J43" s="10"/>
     </row>
     <row r="44" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A44" s="2"/>
-      <c r="B44" s="164"/>
-      <c r="C44" s="170"/>
+      <c r="B44" s="189"/>
+      <c r="C44" s="195"/>
       <c r="D44" s="15" t="s">
         <v>49</v>
       </c>
@@ -4999,14 +4999,14 @@
       <c r="G44" s="16">
         <v>0.40972222222222221</v>
       </c>
-      <c r="H44" s="187"/>
-      <c r="I44" s="133"/>
+      <c r="H44" s="178"/>
+      <c r="I44" s="125"/>
       <c r="J44" s="10"/>
     </row>
     <row r="45" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="2"/>
-      <c r="B45" s="164"/>
-      <c r="C45" s="171"/>
+      <c r="B45" s="189"/>
+      <c r="C45" s="196"/>
       <c r="D45" s="17" t="s">
         <v>49</v>
       </c>
@@ -5019,13 +5019,13 @@
       <c r="G45" s="67">
         <v>0.70138888888888884</v>
       </c>
-      <c r="H45" s="188"/>
-      <c r="I45" s="134"/>
+      <c r="H45" s="179"/>
+      <c r="I45" s="144"/>
       <c r="J45" s="10"/>
     </row>
     <row r="46" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="2"/>
-      <c r="B46" s="164"/>
+      <c r="B46" s="189"/>
       <c r="C46" s="73" t="s">
         <v>42</v>
       </c>
@@ -5051,7 +5051,7 @@
     </row>
     <row r="47" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="2"/>
-      <c r="B47" s="165"/>
+      <c r="B47" s="190"/>
       <c r="C47" s="74" t="s">
         <v>41</v>
       </c>
@@ -5089,6 +5089,12 @@
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="B5:B47"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="C7:C10"/>
+    <mergeCell ref="C11:C34"/>
+    <mergeCell ref="C35:C41"/>
+    <mergeCell ref="C42:C45"/>
     <mergeCell ref="I25:I28"/>
     <mergeCell ref="I30:I31"/>
     <mergeCell ref="I42:I45"/>
@@ -5105,12 +5111,6 @@
     <mergeCell ref="H20:H24"/>
     <mergeCell ref="H25:H28"/>
     <mergeCell ref="H29:H31"/>
-    <mergeCell ref="B5:B47"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="C7:C10"/>
-    <mergeCell ref="C11:C34"/>
-    <mergeCell ref="C35:C41"/>
-    <mergeCell ref="C42:C45"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
@@ -5596,7 +5596,7 @@
         <v>DOM</v>
       </c>
       <c r="B23" s="112">
-        <v>0.70833333333333337</v>
+        <v>0.75</v>
       </c>
       <c r="C23" s="112">
         <v>0.90625</v>
@@ -5617,7 +5617,7 @@
         <v>DOM</v>
       </c>
       <c r="B24" s="112">
-        <v>0.70833333333333337</v>
+        <v>0.75</v>
       </c>
       <c r="C24" s="112">
         <v>0.90625</v>
@@ -5638,7 +5638,7 @@
         <v>DOM</v>
       </c>
       <c r="B25" s="112">
-        <v>0.70833333333333337</v>
+        <v>0.75</v>
       </c>
       <c r="C25" s="112">
         <v>0.90625</v>
@@ -5659,7 +5659,7 @@
         <v>DOM</v>
       </c>
       <c r="B26" s="112">
-        <v>0.70833333333333337</v>
+        <v>0.75</v>
       </c>
       <c r="C26" s="112">
         <v>0.90625</v>
@@ -5680,7 +5680,7 @@
         <v>DOM</v>
       </c>
       <c r="B27" s="112">
-        <v>0.70833333333333337</v>
+        <v>0.75</v>
       </c>
       <c r="C27" s="112">
         <v>0.90625</v>

</xml_diff>